<commit_message>
initial work redoing scope 3
</commit_message>
<xml_diff>
--- a/Excel/8_Fuel_WIP_v03.xlsx
+++ b/Excel/8_Fuel_WIP_v03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866CA9E0-A120-4EAB-BA39-304C801936EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506DE4DC-F294-4DF8-9BB7-CE5C69F86125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1215" yWindow="1110" windowWidth="36900" windowHeight="18960" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="660" yWindow="0" windowWidth="37920" windowHeight="20700" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="187">
   <si>
     <t>Home</t>
   </si>
@@ -2488,6 +2488,143 @@
       </fill>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="0.14999847407452621"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <gradientFill degree="90">
+          <stop position="0">
+            <color theme="0"/>
+          </stop>
+          <stop position="1">
+            <color theme="0" tint="-5.0965910824915313E-2"/>
+          </stop>
+        </gradientFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </top>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -4351,143 +4488,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1" tint="0.14999847407452621"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <gradientFill degree="90">
-          <stop position="0">
-            <color theme="0"/>
-          </stop>
-          <stop position="1">
-            <color theme="0" tint="-5.0965910824915313E-2"/>
-          </stop>
-        </gradientFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </top>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -7524,8 +7524,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6E44059A-C219-4316-A7A0-AD77B0121F06}" name="Table_Input_Fuel" displayName="Table_Input_Fuel" ref="D10:I22" totalsRowDxfId="109" headerRowCellStyle="Input table column header">
-  <autoFilter ref="D10:I22" xr:uid="{6E44059A-C219-4316-A7A0-AD77B0121F06}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6E44059A-C219-4316-A7A0-AD77B0121F06}" name="Table_Input_Fuel" displayName="Table_Input_Fuel" ref="D10:I11" totalsRowDxfId="23" headerRowCellStyle="Input table column header">
+  <autoFilter ref="D10:I11" xr:uid="{6E44059A-C219-4316-A7A0-AD77B0121F06}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -7534,14 +7534,16 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="2" xr3:uid="{9540E705-999C-466B-A6B4-24C60E9153AE}" name="Fuel use (select)" totalsRowFunction="average" totalsRowDxfId="108" dataCellStyle="Input select" totalsRowCellStyle="Input select"/>
-    <tableColumn id="3" xr3:uid="{30909C53-73F3-46FE-93B7-F60E126CD84F}" name="Fuel type (select)" totalsRowDxfId="107" dataCellStyle="Input select" totalsRowCellStyle="Input select"/>
-    <tableColumn id="4" xr3:uid="{9DFFE0DC-C289-47FB-8F0C-2D2F480EEE4C}" name="Amount purchased" totalsRowDxfId="106" totalsRowCellStyle="Content bold"/>
-    <tableColumn id="6" xr3:uid="{29AE264C-132E-48F6-8BA3-262EAF9E4687}" name="Amount unit" totalsRowDxfId="105" dataCellStyle="Input number general calculated" totalsRowCellStyle="Input text calculated"/>
-    <tableColumn id="5" xr3:uid="{B9F0EEB0-BF4E-4AB9-8B4B-25BBC232DE33}" name="Percent consumed" totalsRowDxfId="104" totalsRowCellStyle="Input percent">
+    <tableColumn id="2" xr3:uid="{9540E705-999C-466B-A6B4-24C60E9153AE}" name="Fuel use (select)" totalsRowFunction="average" totalsRowDxfId="22" dataCellStyle="Input select" totalsRowCellStyle="Input select"/>
+    <tableColumn id="3" xr3:uid="{30909C53-73F3-46FE-93B7-F60E126CD84F}" name="Fuel type (select)" totalsRowDxfId="21" dataCellStyle="Input select" totalsRowCellStyle="Input select"/>
+    <tableColumn id="4" xr3:uid="{9DFFE0DC-C289-47FB-8F0C-2D2F480EEE4C}" name="Amount purchased" totalsRowDxfId="20" totalsRowCellStyle="Content bold"/>
+    <tableColumn id="6" xr3:uid="{29AE264C-132E-48F6-8BA3-262EAF9E4687}" name="Amount unit" totalsRowDxfId="19" dataCellStyle="Input number general calculated" totalsRowCellStyle="Input text calculated">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{B9F0EEB0-BF4E-4AB9-8B4B-25BBC232DE33}" name="Percent consumed" totalsRowDxfId="18" totalsRowCellStyle="Input percent">
       <calculatedColumnFormula>1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{AE1D2D8C-400E-46F5-850E-2BBEDF1657F8}" name="Amount consumed" totalsRowFunction="custom" totalsRowDxfId="103" dataCellStyle="Input number general calculated" totalsRowCellStyle="Input number 3 decimal places calculated">
+    <tableColumn id="1" xr3:uid="{AE1D2D8C-400E-46F5-850E-2BBEDF1657F8}" name="Amount consumed" totalsRowFunction="custom" totalsRowDxfId="17" dataCellStyle="Input number general calculated" totalsRowCellStyle="Input number 3 decimal places calculated">
       <calculatedColumnFormula>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table_Input_Fuel[Amount consumed])</totalsRowFormula>
     </tableColumn>
@@ -7636,49 +7638,49 @@
     <tableColumn id="1" xr3:uid="{7C646E3D-156E-438B-9E75-102B5E96E255}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3F6652C3-1BDE-4F33-9D5E-1BA7F24CFE1E}" name="MAT" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{3F6652C3-1BDE-4F33-9D5E-1BA7F24CFE1E}" name="MAT" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{68D3A033-0C56-472E-A3CF-B482905871CF}" name="MAP" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{68D3A033-0C56-472E-A3CF-B482905871CF}" name="MAP" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{18D7CFC5-1F89-47C0-AF12-0FD6A80AD2C8}" name="Frost days per year" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{18D7CFC5-1F89-47C0-AF12-0FD6A80AD2C8}" name="Frost days per year" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{694DED4D-19CA-49A7-A7A4-ED3CD36E0BA2}" name="Elevation" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{694DED4D-19CA-49A7-A7A4-ED3CD36E0BA2}" name="Elevation" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{BE47AD00-59A1-4916-A3FF-4E905492D142}" name="MAP:PET" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{BE47AD00-59A1-4916-A3FF-4E905492D142}" name="MAP:PET" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{8CD0BB0E-B9A0-4065-920B-F859089361EB}" name="Min temp" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{8CD0BB0E-B9A0-4065-920B-F859089361EB}" name="Min temp" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9AD474F5-6F0E-4F15-87EA-A3E86BD8CD84}" name="Max temp" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{9AD474F5-6F0E-4F15-87EA-A3E86BD8CD84}" name="Max temp" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{4132B96D-08DF-47B8-9134-F88DA6CBA26A}" name="Min rainfall" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{4132B96D-08DF-47B8-9134-F88DA6CBA26A}" name="Min rainfall" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{799D2CC4-68A8-4F6B-B5E8-BA9B134CD629}" name="Max rainfall" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{799D2CC4-68A8-4F6B-B5E8-BA9B134CD629}" name="Max rainfall" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FF3C7CFE-CC8F-4407-9CD2-DB7BCF735828}" name="Min frost days" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{FF3C7CFE-CC8F-4407-9CD2-DB7BCF735828}" name="Min frost days" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{9CB12B6D-F283-41CE-A0AC-7DA70F3FEA35}" name="Max frost days" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{9CB12B6D-F283-41CE-A0AC-7DA70F3FEA35}" name="Max frost days" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{DE6B8D57-DEA5-4CDB-BEA5-6794B3B8B4C1}" name="Min elevation" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{DE6B8D57-DEA5-4CDB-BEA5-6794B3B8B4C1}" name="Min elevation" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{F1C5507D-FFFD-4456-AAE0-9309987F0339}" name="Max elevation" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{F1C5507D-FFFD-4456-AAE0-9309987F0339}" name="Max elevation" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{BB91B1DF-4B57-426B-BF6A-71715747D3B2}" name="Min MAP:PET" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{BB91B1DF-4B57-426B-BF6A-71715747D3B2}" name="Min MAP:PET" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{7674CAA3-6E67-48AA-BF62-AECA84F01CB9}" name="Max MAP:PET" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{7674CAA3-6E67-48AA-BF62-AECA84F01CB9}" name="Max MAP:PET" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7696,7 +7698,7 @@
     <tableColumn id="1" xr3:uid="{9DF69629-1C76-40A4-BBA1-FB28BF754268}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{99A9C0E3-7924-426C-A581-5C219452362E}" name="Wet or Dry Zone" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{99A9C0E3-7924-426C-A581-5C219452362E}" name="Wet or Dry Zone" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7802,7 +7804,7 @@
     <tableColumn id="1" xr3:uid="{D0B2F492-E516-47ED-A029-67FEF667A678}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{51E6CA6F-68DC-47AB-A1BB-C75D3CA8FA3B}" name="FracWET" dataDxfId="36">
+    <tableColumn id="2" xr3:uid="{51E6CA6F-68DC-47AB-A1BB-C75D3CA8FA3B}" name="FracWET" dataDxfId="43">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7811,7 +7813,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2781308E-D97C-445B-A805-DE74F822CC4F}" name="Table_Fuel_EFs_StationaryLiquid" displayName="Table_Fuel_EFs_StationaryLiquid" ref="D53:K77" totalsRowShown="0" headerRowDxfId="102" dataDxfId="101">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2781308E-D97C-445B-A805-DE74F822CC4F}" name="Table_Fuel_EFs_StationaryLiquid" displayName="Table_Fuel_EFs_StationaryLiquid" ref="D53:K77" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
   <autoFilter ref="D53:K77" xr:uid="{2781308E-D97C-445B-A805-DE74F822CC4F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -7823,28 +7825,28 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{116B9F07-FAFA-45B6-8BAF-D037C420E4F7}" name="Fuel combusted" dataDxfId="100">
+    <tableColumn id="1" xr3:uid="{116B9F07-FAFA-45B6-8BAF-D037C420E4F7}" name="Fuel combusted" dataDxfId="107">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A9A16324-59CF-4AFF-A845-5DBEFF96AF36}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="99">
+    <tableColumn id="2" xr3:uid="{A9A16324-59CF-4AFF-A845-5DBEFF96AF36}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="106">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D90C1066-FE05-40B0-93E8-B444B2515AC4}" name="Fuel unit" dataDxfId="98">
+    <tableColumn id="3" xr3:uid="{D90C1066-FE05-40B0-93E8-B444B2515AC4}" name="Fuel unit" dataDxfId="105">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{6C9BACBD-72E6-4C6C-8E91-9FC2EE427A52}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="97">
+    <tableColumn id="4" xr3:uid="{6C9BACBD-72E6-4C6C-8E91-9FC2EE427A52}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="104">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9C1D1D67-0EE2-4865-BD1D-E11FDD50B838}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="96">
+    <tableColumn id="5" xr3:uid="{9C1D1D67-0EE2-4865-BD1D-E11FDD50B838}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="103">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{422B50D3-73D6-4895-B780-E80D65DEA437}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="95">
+    <tableColumn id="6" xr3:uid="{422B50D3-73D6-4895-B780-E80D65DEA437}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="102">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3D29A47C-AFAA-45B9-B05D-9137798FA43D}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="94">
+    <tableColumn id="7" xr3:uid="{3D29A47C-AFAA-45B9-B05D-9137798FA43D}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="101">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BA6033AB-70D7-4E8F-B8F8-2A659A19966B}" name="Scope 3 Emission Factor (kg CO2 - e / GJ)" dataDxfId="93">
+    <tableColumn id="8" xr3:uid="{BA6033AB-70D7-4E8F-B8F8-2A659A19966B}" name="Scope 3 Emission Factor (kg CO2 - e / GJ)" dataDxfId="100">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsStationaryLiquid_Data(), Table_Fuel_EFs_StationaryLiquid[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7892,7 +7894,7 @@
     <tableColumn id="1" xr3:uid="{0CAEDF1E-5A86-4C59-ADB4-2A63E7ABD4DD}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{57851871-7E08-4269-B67C-A96E5A947487}" name="FracWET" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{57851871-7E08-4269-B67C-A96E5A947487}" name="FracWET" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7910,7 +7912,7 @@
     <tableColumn id="1" xr3:uid="{04E57D99-757F-4374-BB84-42339A5C3083}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{92543612-DE1F-4C45-B1F2-46B34452C302}" name="EFPRP" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{92543612-DE1F-4C45-B1F2-46B34452C302}" name="EFPRP" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7928,7 +7930,7 @@
     <tableColumn id="1" xr3:uid="{5C54F0C5-3505-4964-A85B-6C95900D28A5}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DE5E22FE-C43A-4172-9EDB-6FE00B1DF854}" name="Season" dataDxfId="33" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DE5E22FE-C43A-4172-9EDB-6FE00B1DF854}" name="Season" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7960,49 +7962,49 @@
     <tableColumn id="1" xr3:uid="{FD606263-AC8F-4B13-96E2-C9CA0ECFC2B3}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{328E4735-CE75-4070-9C88-AE6AC281FA52}" name="MAT (ºC)" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{328E4735-CE75-4070-9C88-AE6AC281FA52}" name="MAT (ºC)" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{AAAA9F18-86A5-4F62-9B13-8EC468FD3268}" name="Anaerobic lagoon" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{AAAA9F18-86A5-4F62-9B13-8EC468FD3268}" name="Anaerobic lagoon" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{16CDDAC7-40E8-4B7E-A5A7-534574EF9960}" name="Digester / covered lagoons" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{16CDDAC7-40E8-4B7E-A5A7-534574EF9960}" name="Digester / covered lagoons" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7BE7531C-242C-4F06-B612-2455D4071B48}" name="Liquid systems" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{7BE7531C-242C-4F06-B612-2455D4071B48}" name="Liquid systems" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4AA6EA91-67D5-4225-8E66-D79949E45C79}" name="Daily spread" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{4AA6EA91-67D5-4225-8E66-D79949E45C79}" name="Daily spread" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{A682CC91-6B5E-45D1-857C-0228079BCC7C}" name="Composting (passive windrow)" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{A682CC91-6B5E-45D1-857C-0228079BCC7C}" name="Composting (passive windrow)" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{516A42DC-F452-4685-9EE1-8DB5323E888F}" name="Solid storage" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{516A42DC-F452-4685-9EE1-8DB5323E888F}" name="Solid storage" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3E59565B-237D-4BF7-8514-8C00EE69787F}" name="Pit storage" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{3E59565B-237D-4BF7-8514-8C00EE69787F}" name="Pit storage" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{B94C989A-1174-49BC-8E63-5C88C372C925}" name="Deep litter" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{B94C989A-1174-49BC-8E63-5C88C372C925}" name="Deep litter" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{4E416B5A-6B9A-4444-8C96-0603C11DC870}" name="Poultry manure with bedding" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{4E416B5A-6B9A-4444-8C96-0603C11DC870}" name="Poultry manure with bedding" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{2302252A-7FB0-4046-9B12-B1CD2F1BBED4}" name="Poultry manure without bedding" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{2302252A-7FB0-4046-9B12-B1CD2F1BBED4}" name="Poultry manure without bedding" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{50CED419-50AF-49B3-8F42-E496D5B781AB}" name="Direct processing" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{50CED419-50AF-49B3-8F42-E496D5B781AB}" name="Direct processing" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{FACDE6F8-8A2F-4040-8D12-2E35D0831482}" name="Direct application" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{FACDE6F8-8A2F-4040-8D12-2E35D0831482}" name="Direct application" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{2134A83A-1EB7-471E-ADAA-05ADE14C7593}" name="Pasture range and paddock" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{2134A83A-1EB7-471E-ADAA-05ADE14C7593}" name="Pasture range and paddock" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{1C3199CA-00F6-4D2D-9A1A-14E5576B6B3A}" name="MAT raw" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{1C3199CA-00F6-4D2D-9A1A-14E5576B6B3A}" name="MAT raw" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8020,7 +8022,7 @@
     <tableColumn id="1" xr3:uid="{6441941C-5801-414B-9EFC-BFCD02E9AABA}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AFFF76A7-AEC2-426D-9FB9-7DCEAE399701}" name="EFNi &amp; EFN2Oi" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AFFF76A7-AEC2-426D-9FB9-7DCEAE399701}" name="EFNi &amp; EFN2Oi" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8029,7 +8031,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{52589EE1-5F69-4B49-BF30-7629445C4436}" name="Table_Fuel_EFs_Transport" displayName="Table_Fuel_EFs_Transport" ref="D9:L34" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{52589EE1-5F69-4B49-BF30-7629445C4436}" name="Table_Fuel_EFs_Transport" displayName="Table_Fuel_EFs_Transport" ref="D9:L34" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
   <autoFilter ref="D9:L34" xr:uid="{52589EE1-5F69-4B49-BF30-7629445C4436}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8042,31 +8044,31 @@
     <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{8D6C44B0-0762-4110-AC2D-7FEE6A4ACB70}" name="Transport type" dataDxfId="90">
+    <tableColumn id="1" xr3:uid="{8D6C44B0-0762-4110-AC2D-7FEE6A4ACB70}" name="Transport type" dataDxfId="97">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3A6969F6-FF37-4AA5-AE1C-FE6AA1A0B2B2}" name="Fuel combusted" dataDxfId="89">
+    <tableColumn id="2" xr3:uid="{3A6969F6-FF37-4AA5-AE1C-FE6AA1A0B2B2}" name="Fuel combusted" dataDxfId="96">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{432B61FE-9A6D-43B7-8616-F6CFE6FB153A}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="88">
+    <tableColumn id="3" xr3:uid="{432B61FE-9A6D-43B7-8616-F6CFE6FB153A}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="95">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{71D7F858-6D97-44C6-8413-957075191C0B}" name="Fuel unit" dataDxfId="87">
+    <tableColumn id="4" xr3:uid="{71D7F858-6D97-44C6-8413-957075191C0B}" name="Fuel unit" dataDxfId="94">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C388B4A9-A36E-4EC9-B5CE-2EA624A56083}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="86">
+    <tableColumn id="8" xr3:uid="{C388B4A9-A36E-4EC9-B5CE-2EA624A56083}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="93">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{4E84DFC1-37C7-4930-B71E-DB7CDCBDD458}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="85">
+    <tableColumn id="9" xr3:uid="{4E84DFC1-37C7-4930-B71E-DB7CDCBDD458}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="92">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA43FF41-AF40-4D8F-8B75-A6223466550A}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="84">
+    <tableColumn id="10" xr3:uid="{BA43FF41-AF40-4D8F-8B75-A6223466550A}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="91">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FBCCF4E4-B3CA-463F-B53D-380ECF4BF688}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="83">
+    <tableColumn id="11" xr3:uid="{FBCCF4E4-B3CA-463F-B53D-380ECF4BF688}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="90">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E2A89F98-94A5-4737-A469-DEAA99554138}" name="Scope 3 Emission Factor (kg CO2 - e / GJ)" dataDxfId="82">
+    <tableColumn id="12" xr3:uid="{E2A89F98-94A5-4737-A469-DEAA99554138}" name="Scope 3 Emission Factor (kg CO2 - e / GJ)" dataDxfId="89">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransport_Data(), Table_Fuel_EFs_Transport[[#Headers],[Transport type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8075,7 +8077,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5CE27F6B-DBAC-48D7-85B3-77E92E77D6C0}" name="Table_FuelTypesPerUse" displayName="Table_FuelTypesPerUse" ref="D130:J139" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5CE27F6B-DBAC-48D7-85B3-77E92E77D6C0}" name="Table_FuelTypesPerUse" displayName="Table_FuelTypesPerUse" ref="D130:J139" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
   <autoFilter ref="D130:J139" xr:uid="{5CE27F6B-DBAC-48D7-85B3-77E92E77D6C0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8086,20 +8088,20 @@
     <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{532D4BA3-A3CE-460F-A250-E2A6690A9C59}" name="Generators" dataDxfId="79"/>
-    <tableColumn id="2" xr3:uid="{6E069153-6950-4C63-9ADE-F4A2F0DF67AF}" name="Power standalone machinery or heating" dataDxfId="78"/>
-    <tableColumn id="3" xr3:uid="{3917BF44-833D-42F1-B3B3-C62FEF76A321}" name="Aviation" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{4F35E2A0-90CD-4AC1-B52F-870485779A73}" name="Cars and light commercial vehicles" dataDxfId="76"/>
-    <tableColumn id="7" xr3:uid="{1651A844-7E2B-435C-A7B4-4B0FFD5577CE}" name="Off-road Agriculture and forestry equipment" dataDxfId="75" dataCellStyle="Content bold"/>
-    <tableColumn id="8" xr3:uid="{FCED622E-3FDD-4E8D-B2D1-E4C99EF7323A}" name="Vessels" dataDxfId="74" dataCellStyle="Content bold"/>
-    <tableColumn id="6" xr3:uid="{1E441AA6-3AB5-4373-8C13-AD2F41D6BA71}" name="General use" dataDxfId="73"/>
+    <tableColumn id="1" xr3:uid="{532D4BA3-A3CE-460F-A250-E2A6690A9C59}" name="Generators" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{6E069153-6950-4C63-9ADE-F4A2F0DF67AF}" name="Power standalone machinery or heating" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{3917BF44-833D-42F1-B3B3-C62FEF76A321}" name="Aviation" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{4F35E2A0-90CD-4AC1-B52F-870485779A73}" name="Cars and light commercial vehicles" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{1651A844-7E2B-435C-A7B4-4B0FFD5577CE}" name="Off-road Agriculture and forestry equipment" dataDxfId="82" dataCellStyle="Content bold"/>
+    <tableColumn id="8" xr3:uid="{FCED622E-3FDD-4E8D-B2D1-E4C99EF7323A}" name="Vessels" dataDxfId="81" dataCellStyle="Content bold"/>
+    <tableColumn id="6" xr3:uid="{1E441AA6-3AB5-4373-8C13-AD2F41D6BA71}" name="General use" dataDxfId="80"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2DFA7F9E-607A-4EC9-89A5-ADF4BF63C858}" name="Table_Fuel_EFs_StationaryGaseous" displayName="Table_Fuel_EFs_StationaryGaseous" ref="D86:J104" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2DFA7F9E-607A-4EC9-89A5-ADF4BF63C858}" name="Table_Fuel_EFs_StationaryGaseous" displayName="Table_Fuel_EFs_StationaryGaseous" ref="D86:J104" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
   <autoFilter ref="D86:J104" xr:uid="{2DFA7F9E-607A-4EC9-89A5-ADF4BF63C858}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8110,25 +8112,25 @@
     <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{576104C6-5F3C-42C2-96A5-3F8A6D95B719}" name="Fuel combusted" dataDxfId="70">
+    <tableColumn id="1" xr3:uid="{576104C6-5F3C-42C2-96A5-3F8A6D95B719}" name="Fuel combusted" dataDxfId="77">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{249B0D76-8ABD-4FA7-AE7E-9500D03E43DD}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="69">
+    <tableColumn id="2" xr3:uid="{249B0D76-8ABD-4FA7-AE7E-9500D03E43DD}" name="Energy Content Factor (GJ per unit of fuel)" dataDxfId="76">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{C67F3A46-C70C-439C-A78F-80B7E5662B6A}" name="Fuel unit" dataDxfId="68">
+    <tableColumn id="3" xr3:uid="{C67F3A46-C70C-439C-A78F-80B7E5662B6A}" name="Fuel unit" dataDxfId="75">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B9C45459-33F6-4505-BE9E-03D5C5B7CF41}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="67">
+    <tableColumn id="4" xr3:uid="{B9C45459-33F6-4505-BE9E-03D5C5B7CF41}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CO2" dataDxfId="74">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{484A6982-10DC-4FC8-9C4C-E978774599C6}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="66">
+    <tableColumn id="5" xr3:uid="{484A6982-10DC-4FC8-9C4C-E978774599C6}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) CH4" dataDxfId="73">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{AEE83219-7CD0-494F-84B0-A8CB1BD0A5FA}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="65">
+    <tableColumn id="6" xr3:uid="{AEE83219-7CD0-494F-84B0-A8CB1BD0A5FA}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) N2O" dataDxfId="72">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3B70B10C-4767-4B84-90B0-F26D20C968BC}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="64">
+    <tableColumn id="7" xr3:uid="{3B70B10C-4767-4B84-90B0-F26D20C968BC}" name="Scope 1 Emission Factor (kg CO2 - e / GJ) Combined gases" dataDxfId="71">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous[[#Headers],[Fuel combusted]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8137,20 +8139,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{7D6CE29D-2354-4FAC-9965-9A66FFA42416}" name="Table_Fuel_EFs_StationaryGaseous34" displayName="Table_Fuel_EFs_StationaryGaseous34" ref="D112:F120" headerRowDxfId="63" totalsRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{7D6CE29D-2354-4FAC-9965-9A66FFA42416}" name="Table_Fuel_EFs_StationaryGaseous34" displayName="Table_Fuel_EFs_StationaryGaseous34" ref="D112:F120" headerRowDxfId="70" totalsRowDxfId="69">
   <autoFilter ref="D112:F120" xr:uid="{7D6CE29D-2354-4FAC-9965-9A66FFA42416}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{ECC6D32E-EE87-4C56-B924-DE2296D3A17A}" name="State or territory" totalsRowDxfId="61">
+    <tableColumn id="1" xr3:uid="{ECC6D32E-EE87-4C56-B924-DE2296D3A17A}" name="State or territory" totalsRowDxfId="68">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope3EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous34[[#Headers],[State or territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0BD20FE8-E5F8-4C9A-BA5E-E08126295979}" name="Scope 3 Emission Factors for Natural Gas (kg CO2 - e / GJ) Metro" totalsRowDxfId="60">
+    <tableColumn id="2" xr3:uid="{0BD20FE8-E5F8-4C9A-BA5E-E08126295979}" name="Scope 3 Emission Factors for Natural Gas (kg CO2 - e / GJ) Metro" totalsRowDxfId="67">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope3EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous34[[#Headers],[State or territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{25FB53B2-D2E0-4CEA-8D3F-87F6DBB9EB6B}" name="Scope 3 Emission Factors for Natural Gas (kg CO2 - e / GJ) Non - Metro" totalsRowDxfId="59">
+    <tableColumn id="3" xr3:uid="{25FB53B2-D2E0-4CEA-8D3F-87F6DBB9EB6B}" name="Scope 3 Emission Factors for Natural Gas (kg CO2 - e / GJ) Non - Metro" totalsRowDxfId="66">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope3EmissionFactorsStationaryGaseous_Data(), Table_Fuel_EFs_StationaryGaseous34[[#Headers],[State or territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8187,22 +8189,22 @@
     <tableColumn id="1" xr3:uid="{4C846971-D1AE-40B6-93C3-4B2219305A91}" name="Transport type t">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{82F6DC4A-0F92-4452-8487-4E43D14ADFD1}" name="Fuel type q" dataDxfId="58" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{82F6DC4A-0F92-4452-8487-4E43D14ADFD1}" name="Fuel type q" dataDxfId="65" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3C4A929E-9ED1-4901-B86F-83D8164C35AA}" name="ECTrans,q (GJ/kL)" dataDxfId="57" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{3C4A929E-9ED1-4901-B86F-83D8164C35AA}" name="ECTrans,q (GJ/kL)" dataDxfId="64" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{CC9C9248-897D-415C-976A-2C740F057EB1}" name="Scope 1 CO2 EFTran,1,tqg (kg CO2-e/GJ)" dataDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{CC9C9248-897D-415C-976A-2C740F057EB1}" name="Scope 1 CO2 EFTran,1,tqg (kg CO2-e/GJ)" dataDxfId="63" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{786BC3D5-A6A8-43D0-B256-FFFC5437A688}" name="Scope 1 CH4 EFTran,1,tgg (kg CO2-e/GJ)" dataDxfId="55" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{786BC3D5-A6A8-43D0-B256-FFFC5437A688}" name="Scope 1 CH4 EFTran,1,tgg (kg CO2-e/GJ)" dataDxfId="62" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{6D5BCB7A-89DA-40E3-B7CA-1C29764B596B}" name="Scope 1 N2O EFTran,1,tgg (kg CO2-e/GJ)" dataDxfId="54" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{6D5BCB7A-89DA-40E3-B7CA-1C29764B596B}" name="Scope 1 N2O EFTran,1,tgg (kg CO2-e/GJ)" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7E1DA076-D5F8-4B6F-B281-1DB030412A87}" name="Scope 3 EFTrans,3,q (kg CO2-e/GJ)" dataDxfId="53" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{7E1DA076-D5F8-4B6F-B281-1DB030412A87}" name="Scope 3 EFTrans,3,q (kg CO2-e/GJ)" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Fuel_SourceData.Fuel_Scope1Scope3EmissionFactorsTransportOffRoad_Data(), Table_SourceData_Fuel_TransportOffroad[[#Headers],[Transport type t]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8959,11 +8961,11 @@
       </c>
       <c r="E15" s="65">
         <f>'8.X.1.1-2 General use fuel'!E36</f>
-        <v>1.1287170000000002</v>
+        <v>0.23050800000000005</v>
       </c>
       <c r="F15" s="65">
         <f t="shared" si="0"/>
-        <v>1.1287170000000002</v>
+        <v>0.23050800000000005</v>
       </c>
       <c r="G15" s="33" t="s">
         <v>59</v>
@@ -8981,11 +8983,11 @@
       </c>
       <c r="E16" s="65">
         <f>'8.X.1.1-2 General use fuel'!E37</f>
-        <v>6.8774499999999994E-3</v>
+        <v>3.7620000000000004E-4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" si="0"/>
-        <v>6.8774499999999994E-3</v>
+        <v>3.7620000000000004E-4</v>
       </c>
       <c r="G16" s="33" t="s">
         <v>59</v>
@@ -9003,11 +9005,11 @@
       </c>
       <c r="E17" s="65">
         <f>'8.X.1.1-2 General use fuel'!E38</f>
-        <v>1.4673749999999999E-2</v>
+        <v>6.8400000000000015E-4</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" si="0"/>
-        <v>1.4673749999999999E-2</v>
+        <v>6.8400000000000015E-4</v>
       </c>
       <c r="G17" s="33" t="s">
         <v>59</v>
@@ -9021,11 +9023,11 @@
       </c>
       <c r="E18" s="46">
         <f>SUM(E9:E17)</f>
-        <v>1.1502682000000002</v>
+        <v>0.23156820000000003</v>
       </c>
       <c r="F18" s="46">
         <f>SUM(F9:F17)</f>
-        <v>1.1502682000000002</v>
+        <v>0.23156820000000003</v>
       </c>
       <c r="G18" s="44" t="s">
         <v>59</v>
@@ -9594,7 +9596,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC610A2-02A7-4F78-A2BB-B4DFE856D1FB}">
-  <dimension ref="A1:J361"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -9747,103 +9749,19 @@
         <f>HYPERLINK("#'8.2.1.1-2 Stationary fuel'!A1", "8.2.1.1-2 Stationary fuel")</f>
         <v>8.2.1.1-2 Stationary fuel</v>
       </c>
-      <c r="D12" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="F12" s="73">
-        <v>100</v>
-      </c>
-      <c r="G12" s="31" t="str" cm="1">
-        <f t="array" ref="G12">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H12" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I12" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
     </row>
     <row r="13" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="str">
         <f>HYPERLINK("#'8.X.1.1-2 General use fuel'!A1", "8.X.1.1-2 General use fuel")</f>
         <v>8.X.1.1-2 General use fuel</v>
       </c>
-      <c r="D13" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F13" s="73">
-        <v>100</v>
-      </c>
-      <c r="G13" s="31" t="str" cm="1">
-        <f t="array" ref="G13">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H13" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I13" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
     </row>
     <row r="14" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
-      <c r="D14" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="F14" s="73">
-        <v>100</v>
-      </c>
-      <c r="G14" s="31" t="str" cm="1">
-        <f t="array" ref="G14">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H14" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I14" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
     </row>
     <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>2</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="F15" s="73">
-        <v>100</v>
-      </c>
-      <c r="G15" s="31" t="str" cm="1">
-        <f t="array" ref="G15">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H15" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I15" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9851,190 +9769,40 @@
         <f>HYPERLINK("#'Constants - Fuel'!A1", "Constants - Fuel")</f>
         <v>Constants - Fuel</v>
       </c>
-      <c r="D16" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F16" s="73">
-        <v>100</v>
-      </c>
-      <c r="G16" s="31" t="str" cm="1">
-        <f t="array" ref="G16">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H16" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I16" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="str">
         <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
         <v>Constants - Common</v>
       </c>
-      <c r="D17" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="F17" s="73">
-        <v>100</v>
-      </c>
-      <c r="G17" s="31" t="str" cm="1">
-        <f t="array" ref="G17">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H17" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I17" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="F18" s="73">
-        <v>100</v>
-      </c>
-      <c r="G18" s="31" t="str" cm="1">
-        <f t="array" ref="G18">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H18" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I18" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="F19" s="73">
-        <v>100</v>
-      </c>
-      <c r="G19" s="31" t="str" cm="1">
-        <f t="array" ref="G19">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H19" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I19" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
-      <c r="D20" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="F20" s="73">
-        <v>100</v>
-      </c>
-      <c r="G20" s="31" t="str" cm="1">
-        <f t="array" ref="G20">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>kL</v>
-      </c>
-      <c r="H20" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I20" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14"/>
-      <c r="D21" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="F21" s="73">
-        <v>100</v>
-      </c>
-      <c r="G21" s="31" t="str" cm="1">
-        <f t="array" ref="G21">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>GJ</v>
-      </c>
-      <c r="H21" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I21" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" s="73">
-        <v>100</v>
-      </c>
-      <c r="G22" s="31" t="str" cm="1">
-        <f t="array" ref="G22">Common_InputFunctions.Utility_LookupValueInTable(Table_Input_Fuel[[#This Row],[Fuel type (select)]],Table_FuelTypes_Units[Fuel type], Table_FuelTypes_Units[Unit])</f>
-        <v>GJ</v>
-      </c>
-      <c r="H22" s="74">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="I22" s="31">
-        <f>Table_Input_Fuel[[#This Row],[Amount purchased]]*Table_Input_Fuel[[#This Row],[Percent consumed]]*10^-3</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14"/>
     </row>
-    <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
     </row>
-    <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
     </row>
-    <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="35"/>
     </row>
-    <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="35"/>
     </row>
     <row r="33" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -10200,122 +9968,122 @@
     <row r="163" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="164" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="165" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="361" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D361" s="45"/>
+    <row r="350" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D350" s="45"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F47">
+  <conditionalFormatting sqref="F36">
     <cfRule type="cellIs" dxfId="16" priority="62" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F126:F127">
+  <conditionalFormatting sqref="F115:F116">
     <cfRule type="cellIs" dxfId="15" priority="21" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F138:F139">
+  <conditionalFormatting sqref="F127:F128">
     <cfRule type="cellIs" dxfId="14" priority="20" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F150:F151">
+  <conditionalFormatting sqref="F139:F140">
     <cfRule type="cellIs" dxfId="13" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F162:F163">
+  <conditionalFormatting sqref="F151:F152">
     <cfRule type="cellIs" dxfId="12" priority="18" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F250:F251">
+  <conditionalFormatting sqref="F239:F240">
     <cfRule type="cellIs" dxfId="11" priority="93" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F255:F256">
+  <conditionalFormatting sqref="F244:F245">
     <cfRule type="cellIs" dxfId="10" priority="92" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F260:F261">
+  <conditionalFormatting sqref="F249:F250">
     <cfRule type="cellIs" dxfId="9" priority="91" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F284:F285">
+  <conditionalFormatting sqref="F273:F274">
     <cfRule type="cellIs" dxfId="8" priority="85" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F289:F290">
+  <conditionalFormatting sqref="F278:F279">
     <cfRule type="cellIs" dxfId="7" priority="84" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F294:F295">
+  <conditionalFormatting sqref="F283:F284">
     <cfRule type="cellIs" dxfId="6" priority="83" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I31 I33:I37 I41:I42 H43:H45 I46 I48:I50 I52:I53 I204 E210:G210 I210">
+  <conditionalFormatting sqref="I20 I22:I26 I30:I31 H32:H34 I35 I37:I39 I41:I42 I193 E199:G199 I199">
     <cfRule type="cellIs" dxfId="5" priority="79" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I57:I61">
+  <conditionalFormatting sqref="I46:I50">
     <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I65 I124">
+  <conditionalFormatting sqref="I54 I113">
     <cfRule type="cellIs" dxfId="3" priority="74" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I76:I78">
+  <conditionalFormatting sqref="I65:I67">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I82:I85">
+  <conditionalFormatting sqref="I71:I74">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I89:I93">
+  <conditionalFormatting sqref="I78:I82">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D277" xr:uid="{4E913AB3-F90B-4C35-BCE1-5DBB8FC05107}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D266" xr:uid="{4E913AB3-F90B-4C35-BCE1-5DBB8FC05107}">
       <formula1>INDIRECT("Table_SourceData_PoultryMMSStage1[MMS]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E225" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E214" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
       <formula1>INDIRECT("Table_SourceData_Dairy_ProductionSystemTemplates[Area]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E249 E254 E259 E293 E288 E283 E161 E149 E125 E137" xr:uid="{00A4EA4C-90D3-4150-979D-4D71C7F37A31}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E238 E243 E248 E282 E277 E272 E150 E138 E114 E126" xr:uid="{00A4EA4C-90D3-4150-979D-4D71C7F37A31}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E65" xr:uid="{DBA884B0-B52E-420E-8FD2-21B082EB75E2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E54" xr:uid="{DBA884B0-B52E-420E-8FD2-21B082EB75E2}">
       <formula1>INDIRECT("Table_SourceData_Swine_IrrigationMethods[Irrigation method]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E64" xr:uid="{B95E29DC-96D0-4475-A29E-3F3A3B60CEA1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E53" xr:uid="{B95E29DC-96D0-4475-A29E-3F3A3B60CEA1}">
       <formula1>INDIRECT("Table_SourceData_Swine_CropProdSystems[Production system]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H24:H25" xr:uid="{4A7ED0FB-DC6D-4B9E-B043-37B0C0BD600A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H13:H14" xr:uid="{4A7ED0FB-DC6D-4B9E-B043-37B0C0BD600A}">
       <formula1>INDIRECT("Table_Fertiliser_ChemicalCompounds[Fertiliser type f]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D44:D45" xr:uid="{23F8C720-A764-46DD-9B01-B7EA3D86E5AB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D33:D34" xr:uid="{23F8C720-A764-46DD-9B01-B7EA3D86E5AB}">
       <formula1>INDIRECT("Table_SourceData_OrganicFertiliserTypes[Organic fertiliser type]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E22" xr:uid="{76773934-728A-4512-A789-D38AF73B28FA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11" xr:uid="{44BCE1B2-993E-4D7C-8172-C366FD07D726}">
+      <formula1>INDIRECT("Table_FuelTypesPerUse[#Headers]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11" xr:uid="{76773934-728A-4512-A789-D38AF73B28FA}">
       <formula1>_xlfn.TRIMRANGE(INDIRECT("Table_FuelTypesPerUse["&amp;D11&amp;"]"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11:D22" xr:uid="{44BCE1B2-993E-4D7C-8172-C366FD07D726}">
-      <formula1>INDIRECT("Table_FuelTypesPerUse[#Headers]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14029,7 +13797,7 @@
       </c>
       <c r="K25" s="64" cm="1">
         <f t="array" ref="K25">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D25, Table_Input_Fuel[Fuel type (select)],F25)</f>
-        <v>0.30000000000000004</v>
+        <v>0.1</v>
       </c>
       <c r="L25" s="64" t="str" cm="1">
         <f t="array" ref="L25">Common_InputFunctions.Utility_LookupValueInTable(F25,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14037,15 +13805,15 @@
       </c>
       <c r="M25" s="107" cm="1">
         <f t="array" ref="M25">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K25,$G25,H25)</f>
-        <v>0.69152400000000014</v>
+        <v>0.23050800000000005</v>
       </c>
       <c r="N25" s="107" cm="1">
         <f t="array" ref="N25">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K25,$G25,I25)</f>
-        <v>1.1286000000000002E-3</v>
+        <v>3.7620000000000004E-4</v>
       </c>
       <c r="O25" s="107" cm="1">
         <f t="array" ref="O25">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K25,$G25,J25)</f>
-        <v>2.0520000000000004E-3</v>
+        <v>6.8400000000000015E-4</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14079,7 +13847,7 @@
       </c>
       <c r="K26" s="64" cm="1">
         <f t="array" ref="K26">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D26, Table_Input_Fuel[Fuel type (select)],F26)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L26" s="64" t="str" cm="1">
         <f t="array" ref="L26">Common_InputFunctions.Utility_LookupValueInTable(F26,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14087,15 +13855,15 @@
       </c>
       <c r="M26" s="107" cm="1">
         <f t="array" ref="M26">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K26,$G26,H26)</f>
-        <v>0.26981400000000005</v>
+        <v>0</v>
       </c>
       <c r="N26" s="107" cm="1">
         <f t="array" ref="N26">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K26,$G26,I26)</f>
-        <v>2.1230000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="O26" s="107" cm="1">
         <f t="array" ref="O26">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K26,$G26,J26)</f>
-        <v>1.351E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14129,7 +13897,7 @@
       </c>
       <c r="K27" s="64" cm="1">
         <f t="array" ref="K27">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D27, Table_Input_Fuel[Fuel type (select)],F27)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="64" t="str" cm="1">
         <f t="array" ref="L27">Common_InputFunctions.Utility_LookupValueInTable(F27,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14137,15 +13905,15 @@
       </c>
       <c r="M27" s="107" cm="1">
         <f t="array" ref="M27">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K27,$G27,H27)</f>
-        <v>0.15621900000000002</v>
+        <v>0</v>
       </c>
       <c r="N27" s="107" cm="1">
         <f t="array" ref="N27">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K27,$G27,I27)</f>
-        <v>9.0824999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="O27" s="107" cm="1">
         <f t="array" ref="O27">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K27,$G27,J27)</f>
-        <v>6.4875000000000002E-4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14179,7 +13947,7 @@
       </c>
       <c r="K28" s="64" cm="1">
         <f t="array" ref="K28">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D28, Table_Input_Fuel[Fuel type (select)],F28)</f>
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L28" s="64" t="str" cm="1">
         <f t="array" ref="L28">Common_InputFunctions.Utility_LookupValueInTable(F28,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14191,11 +13959,11 @@
       </c>
       <c r="N28" s="107" cm="1">
         <f t="array" ref="N28">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K28,$G28,I28)</f>
-        <v>3.0448000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="O28" s="107" cm="1">
         <f t="array" ref="O28">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K28,$G28,J28)</f>
-        <v>6.5740000000000008E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14229,7 +13997,7 @@
       </c>
       <c r="K29" s="64" cm="1">
         <f t="array" ref="K29">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D29, Table_Input_Fuel[Fuel type (select)],F29)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L29" s="64" t="str" cm="1">
         <f t="array" ref="L29">Common_InputFunctions.Utility_LookupValueInTable(F29,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14241,11 +14009,11 @@
       </c>
       <c r="N29" s="107" cm="1">
         <f t="array" ref="N29">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K29,$G29,I29)</f>
-        <v>3.2759999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="O29" s="107" cm="1">
         <f t="array" ref="O29">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K29,$G29,J29)</f>
-        <v>4.6799999999999999E-4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14279,7 +14047,7 @@
       </c>
       <c r="K30" s="64" cm="1">
         <f t="array" ref="K30">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D30, Table_Input_Fuel[Fuel type (select)],F30)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L30" s="64" t="str" cm="1">
         <f t="array" ref="L30">Common_InputFunctions.Utility_LookupValueInTable(F30,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14291,11 +14059,11 @@
       </c>
       <c r="N30" s="107" cm="1">
         <f t="array" ref="N30">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K30,$G30,I30)</f>
-        <v>1.0295999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="O30" s="107" cm="1">
         <f t="array" ref="O30">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K30,$G30,J30)</f>
-        <v>2.2229999999999997E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14329,7 +14097,7 @@
       </c>
       <c r="K31" s="31" cm="1">
         <f t="array" ref="K31">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D31, Table_Input_Fuel[Fuel type (select)],F31)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L31" s="31" t="str" cm="1">
         <f t="array" ref="L31">Common_InputFunctions.Utility_LookupValueInTable(F31,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14341,11 +14109,11 @@
       </c>
       <c r="N31" s="31" cm="1">
         <f t="array" ref="N31">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K31,$G31,I31)</f>
-        <v>2.1230000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="O31" s="31" cm="1">
         <f t="array" ref="O31">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K31,$G31,J31)</f>
-        <v>1.351E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14379,7 +14147,7 @@
       </c>
       <c r="K32" s="31" cm="1">
         <f t="array" ref="K32">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D32, Table_Input_Fuel[Fuel type (select)],F32)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="31" t="str" cm="1">
         <f t="array" ref="L32">Common_InputFunctions.Utility_LookupValueInTable(F32,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14387,15 +14155,15 @@
       </c>
       <c r="M32" s="31" cm="1">
         <f t="array" ref="M32">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K32,$G32,H32)</f>
-        <v>5.1400000000000005E-3</v>
+        <v>0</v>
       </c>
       <c r="N32" s="31" cm="1">
         <f t="array" ref="N32">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K32,$G32,I32)</f>
-        <v>1.0000000000000003E-5</v>
+        <v>0</v>
       </c>
       <c r="O32" s="31" cm="1">
         <f t="array" ref="O32">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K32,$G32,J32)</f>
-        <v>3.0000000000000001E-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14429,7 +14197,7 @@
       </c>
       <c r="K33" s="31" cm="1">
         <f t="array" ref="K33">Fuel_InputFunctions.Fuel_TotalConsumption(Table_Input_Fuel[Amount consumed], Table_Input_Fuel[Fuel use (select)], D33, Table_Input_Fuel[Fuel type (select)],F33)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L33" s="31" t="str" cm="1">
         <f t="array" ref="L33">Common_InputFunctions.Utility_LookupValueInTable(F33,Table_FuelTypes_Units[Fuel type],Table_FuelTypes_Units[Unit])</f>
@@ -14437,15 +14205,15 @@
       </c>
       <c r="M33" s="31" cm="1">
         <f t="array" ref="M33">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K33,$G33,H33)</f>
-        <v>6.0200000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="N33" s="31" cm="1">
         <f t="array" ref="N33">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K33,$G33,I33)</f>
-        <v>3.9999999999999998E-6</v>
+        <v>0</v>
       </c>
       <c r="O33" s="31" cm="1">
         <f t="array" ref="O33">Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary($K33,$G33,J33)</f>
-        <v>3.0000000000000001E-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14468,7 +14236,7 @@
       </c>
       <c r="E36" s="106">
         <f>SUM(M25:M33)</f>
-        <v>1.1287170000000002</v>
+        <v>0.23050800000000005</v>
       </c>
       <c r="F36" s="2" t="str">
         <f>$E$12</f>
@@ -14481,7 +14249,7 @@
       </c>
       <c r="E37" s="106">
         <f>SUM(N25:N33)</f>
-        <v>6.8774499999999994E-3</v>
+        <v>3.7620000000000004E-4</v>
       </c>
       <c r="F37" s="2" t="str">
         <f t="shared" ref="F37:F38" si="1">$E$12</f>
@@ -14498,7 +14266,7 @@
       </c>
       <c r="E38" s="106">
         <f>SUM(O25:O33)</f>
-        <v>1.4673749999999999E-2</v>
+        <v>6.8400000000000015E-4</v>
       </c>
       <c r="F38" s="2" t="str">
         <f t="shared" si="1"/>
@@ -22803,10 +22571,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzACAAaQBuAGMAbAB1AGQAaQBuAGcAIABsAGkAcQB1AGUAZgBpAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgACAAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA1AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAANwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAHUAZQBsACAAYwBvAG0AYgB1AHMAdABlAGQAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABDAG8AbgB0AGUAbgB0ACAARgBhAGMAdABvAHIAIAAoAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwAKQBcACIALAAgAFwAIgBGAHUAZQBsACAAdQBuAGkAdABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAE8AMgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAEgANABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOADIATwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAG8AbQBiAGkAbgBlAGQAIABnAGEAcwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIAAwAC4AMAAzADcANwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADAALgAyACwAIAAwAC4AMAAzACwAIAA1ADEALgA2ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AYQBsACAAbQBpAG4AZQAgAHcAYQBzAHQAZQAgAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4AOQAsACAANAAuADYALAAgADAALgAzACwAIAA1ADYALgA4ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcAByAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAoAHIAZQB2AGUAcgB0AGkAbgBnACAAdABvACAAcwB0AGEAbgBkAGEAcgBkACAAYwBvAG4AZABpAHQAaQBvAG4AcwApAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVQBuAHAAcgBvAGMAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAA2ADIAOQAsACAAXAAiAG0AMwBcACIALAAgADUANgAuADUALAAgADAALgAwADMALAAgADAALgAwADMALAAgADUANgAuADUANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBrAGUAIABvAHYAZQBuACAAZwBhAHMAXAAiACwAIAAwAC4AMAAxADgAMQAsACAAXAAiAG0AMwBcACIALAAgADMANwAuADAALAAgADAALgAwADMALAAgADAALgAwADUALAAgADMANwAuADAAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAbABhAHMAdAAgAGYAdQByAG4AYQBjAGUAIABnAGEAcwBcACIALAAgADAALgAwADAANAAwACwAIABcACIAbQAzAFwAIgAsACAAMgAzADQALgAwACwAIAAwAC4AMAAzACwAIAAwAC4AMAAyACwAIAAyADMANAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwBcACIALAAgADAALgAwADMAOQAwACwAIABcACIAbQAzAFwAIgAsACAANgAwAC4AMgAsACAAMAAuADAANAAsACAAMAAuADAAMwAsACAANgAwAC4AMgA3ADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBMAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAGUAbwB1AHMAIABmAG8AcwBzAGkAbAAgAGYAdQBlAGwAcwAgAG8AdABoAGUAcgAgAHQAaABhAG4AIAB0AGgAbwBzAGUAIABtAGUAbgB0AGkAbwBuAGUAZAAgAGkAbgAgAHQAaABlACAAaQB0AGUAbQBzACAAYQBiAG8AdgBlAFwAIgAsACAAMAAuADAAMwA5ADAALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsACAAYgBpAG8AZwBhAHMAIAB0AGgAYQB0ACAAaQBzACAAYwBhAHAAdAB1AHIAZQBkACAAZgBvAHIAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAKABtAGUAdABoAGEAbgBlACAAbwBuAGwAeQApAFwAIgAsACAAMAAuADAAMwA3ADcALAAgAFwAIgBtADMAXAAiACwAIAAwAC4AMAAsACAANgAuADQALAAgADAALgAwADMALAAgADYALgA0ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgACgAbQBlAHQAaABhAG4AZQAgAG8AbgBsAHkAKQBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADYALgA0ACwAIAAwAC4AMAAzACwAIAA2AC4ANAAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAsACAAbwB0AGgAZQByACAAdABoAGEAbgAgAHQAaABvAHMAZQAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAwAC4AMAAzADcAMAAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAA2AC4ANAAsACAAMAAuADAAMwAsACAANgAuADQAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAG0AZQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAAMAAuADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAeQBkAHIAbwBnAGUAbgBcACIALAAgADAALgAwADEAMgAyACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADAALgAwACwAIAAwAC4ANQAsACAAMAAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdAB1AHIAYQBsACAAZwBhAHMAIABkAGkAcwB0AHIAaQBiAHUAdABlAGQAIABpAG4AIABhACAAcABpAHAAZQBsAGkAbgBlACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAXAAiACwAIAAxACwAIABcACIARwBKAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzAFwAIgAsACAAMQAsACAAXAAiAEcASgBcACIALAAgADYAMAAuADIALAAgADAALgAwADQALAAgADAALgAwADMALAAgADYAMAAuADIANwBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgACcATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzACcAIABhAG4AZAAgACcAVABvAHcAbgAgAGcAYQBzACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAJwAgAHcAZQByAGUAIABhAGQAZABlAGQALAAgAGUAYQBjAGgAIAB3AGkAdABoACAAYQBuACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABvAGYAIAAxACAARwBKACAAcABlAHIAIAB1AG4AaQB0ACAAbwBmACAAZgB1AGUAbAAuACAAVABoAGkAcwAgAGkAcwAgAGYAbwByACAAdQBzAGUAcgBzACAAdwBoAG8AIABoAGEAdgBlACAAZgB1AGUAbAAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGQAYQB0AGEAIABpAG4AIABHAEoAIAByAGEAdABoAGUAcgAgAHQAaABhAG4AIABtADMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGcAYQBzAGUAbwB1AHMAIABmAHUAZQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBGAHUAZQBsACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGcAYQBzAGUAbwB1AHMAIABmAHUAZQBsAHMAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMALgBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADYAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAB0AGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgAGYAbwByACAATgBhAHQAdQByAGEAbAAgAEcAYQBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATQBlAHQAcgBvAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgBzACAAZgBvAHIAIABOAGEAdAB1AHIAYQBsACAARwBhAHMAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOAG8AbgAgAC0AIABNAGUAdAByAG8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIAAxADMALgAxACwAIAAxADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBDAFQAXAAiACwAIAAxADMALgAxACwAIAAxADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAANAAuADAALAAgADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgADgALgA4ACwAIAA3AC4AOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAMQAwAC4ANwAsACAAMQAwAC4ANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADQALgAxACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgADQALgAwACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAANAAuADEALAAgADQALgAwAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATgBTAFcAIABhAG4AZAAgAEEAQwBUACAAcwBwAGwAaQB0ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAHIAbwB3AHMALgAgACcAQwAnACAAVgBhAGwAdQBlAHMAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAGEAbgBkACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAByAGUAcABsAGEAYwBlAGQAIAB3AGkAdABoACAAdABoAG8AcwBlACAAZgBvAHIAIABWAGkAYwB0AG8AcgBpAGEAIABhAG4AZAAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAHIAZQBzAHAAZQBjAHQAaQB2AGUAbAB5AC4AIAAoAFMAZQBlACAAYQBwAHAAZQBuAGQAaQBjAGUAcwApAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEEAcwAgAFMAYwBvAHAAZQAgADMAIABmAGEAYwB0AG8AcgBzACAAYQByAGUAIABjAGEAbABjAHUAbABhAHQAZQBkACAAYQB0ACAAdABoAGUAIABwAG8AaQBuAHQAIAB3AGgAZQByAGUAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIABpAHMAIABkAGUAbABpAHYAZQByAGUAZAAgAHQAbwAgAGUAbgBkACAAdQBzAGUAcgBzACwAIABpAHQAIABpAHMAIABuAGUAYwBlAHMAcwBhAHIAeQAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAYQB0ACAAZQBhAGMAaAAgAG8AZgAgAHQAaABlACAAbABvAGEAZAAgAGMAZQBuAHQAcgBlAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBHAGEAcwAgAHIAZQBhAGMAaABlAHMAIABlAG4AZAAgAHUAcwBlAHIAcwAgAGUAaQB0AGgAZQByACAAZgByAG8AbQAgAHQAaABlACAAbQBlAHQAcgBvACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABuAGUAdAB3AG8AcgBrAHMAIABvAHIAIABkAGkAcgBlAGMAdAAgAGYAcgBvAG0AIAB0AGgAZQAgAGgAaQBnAGgAIAAtACAAcAByAGUAcwBzAHUAcgBlACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABwAGkAcABlAGwAaQBuAGUAcwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAEgAbwB1AHMAZQBoAG8AbABkAHMAIABhAG4AZAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB1AHMAZQByAHMAIAB0AGUAbgBkACAAdABvACAAYgBlACAAcwBlAHIAdgBlAGQAIABiAHkAIAB0AGgAZQAgAGYAbwByAG0AZQByACwAIABhAG4AZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAGcAZQBuAGUAcgBhAHQAbwByAHMAIABhAG4AZAAgAGwAYQByAGcAZQAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIABwAGwAYQBuAHQAcwAgAGYAcgBvAG0AIAB0AGgAZQAgAGwAYQB0AHQAZQByAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBNAGUAdAByAG8AIABpAHMAIABkAGUAZgBpAG4AZQBkACAAYQBzACAAbABvAGMAYQB0AGUAZAAgAG8AbgAgAG8AcgAgAGUAYQBzAHQAIABvAGYAIAB0AGgAZQAgAGQAaQB2AGkAZABpAG4AZwAgAHIAYQBuAGcAZQAgAGkAbgAgAE4AUwBXACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAEMAYQBuAGIAZQByAHIAYQAgAGEAbgBkACAAUQB1AGUAYQBuAGIAZQB5AGEAbgAsACAATQBlAGwAYgBvAHUAcgBuAGUALAAgAEIAcgBpAHMAYgBhAG4AZQAsACAAQQBkAGUAbABhAGkAZABlACAAbwByACAAUABlAHIAdABoAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIATwB0AGgAZQByAHcAaQBzAGUALAAgAHQAaABlACAAbgBvAG4AIAAtACAAbQBlAHQAcgBvACAAZgBhAGMAdABvAHIAIABzAGgAbwB1AGwAZAAgAGIAZQAgAHUAcwBlAGQALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEYAYQBjAHQAbwByAHMAIABhAHIAZQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAGEAbABsACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAHcAaABpAGMAaAAgAG0AYQB5ACAAaQBuAGMAbAB1AGQAZQAgAGMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACwAIABcACIAVABhAGIAbABlACAANgAgAGkAcwAgAG4AbwB0ACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHQAbwAgAGUAdABoAGEAbgBlAC4AIABTAGUAZQAgAFQAYQBiAGwAZQAgADcAIABJAG4AZABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAZQB0AGgAYQBuAGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEMAIAA9ACAAQwBvAG4AZgBpAGQAZQBuAHQAaQBhAGwALgAgAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABUAGEAcwBtAGEAbgBpAGEAIABhAG4AZAAgAHQAaABlACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIABhAHIAZQAgAG4AbwB0ACAAYQB2AGEAaQBsAGEAYgBsAGUAIABkAHUAZQAgAHQAbwAgAGMAbwBuAGYAaQBkAGUAbgB0AGkAYQBsAGkAdAB5ACAAYwBvAG4AcwB0AHIAYQBpAG4AdABzACAAdABoAGEAdAAgAGEAcgBpAHMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBmAHIAbwBtACAAdABoAGUAIAB1AHMAZQAgAG8AZgAgAGEAIABsAGkAbQBpAHQAZQBkACAAbgB1AG0AYgBlAHIAIABvAGYAIABOAEcARQBSACAAZABhAHQAYQAgAGkAbgBwAHUAdABzAC4AIABJAHQAIABpAHMAIABzAHUAZwBnAGUAcwB0AGUAZAAgAHQAaABhAHQAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAHQAaABlACAAdQBzAGUAIABvAGYAIAB0AGgAZQAgAFYAaQBjAHQAbwByAGkAYQBuACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGkAcwAgAGEAcABwAHIAbwBwAHIAaQBhAHQAZQAsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAHcAaABpAGwAZQAgAGYAbwByACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAB0AGgAZQAgAHUAcwBlACAAbwBmACAAdABoAGUAIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABpAHMAIABhAHAAcAByAG8AcAByAGkAYQB0AGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZABvACAAbgBvAHQAIABpAG4AYwBsAHUAZABlACAAZgB1AGcAaQB0AGkAdgBlACAAZQBtAGkAcwBzAGkAbwBuACAAbABlAGEAawBhAGcAZQAgAGYAcgBvAG0AIABsAG8AdwAgAHAAcgBlAHMAcwB1AHIAZQAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGkAbwBuACAAcABpAHAAZQBsAGkAbgBlACAAbgBlAHQAdwBvAHIAawBzACAAdwBoAGkAbABlACAAdABoAG8AcwBlACAAZgByAG8AbQAgAGgAaQBnAGgAIABwAHIAZQBzAHMAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAZwBhAHMAIABuAGUAdAB3AG8AcgBrAHMAIABhAHIAZQAgAGMAbwBuAHMAaQBkAGUAcgBlAGQAIABuAGUAZwBsAGkAZwBpAGIAbABlAC4AXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABTAHQAYQB0AGkAbwBuAGEAcgB5ACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAYQBuAGQAIABpAG4AZABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMALAAgAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBlAHIAdABhAGkAbgAgAHAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMALgBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA4AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADUALAAgADgALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACAAKABHAEoAIABwAGUAcgAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsACkAXAAiACwAIABcACIARgB1AGUAbAAgAHUAbgBpAHQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBPADIAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBIADQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgAyAE8AXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBvAG0AYgBpAG4AZQBkACAAZwBhAHMAZQBzAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsAHMAIAAoAG8AdABoAGUAcgAgAHQAaABhAG4AIABwAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsACAAdQBzAGUAZAAgAGEAcwAgAGYAdQBlAGwAKQAsACAAZQAuAGcALgAgAGwAdQBiAHIAaQBjAGEAbgB0AHMAXAAiACwAIAAzADgALgA4ACwAIABcACIAawBsAFwAIgAsACAAMQAzAC4AOQAsACAAMAAuADAALAAgADAALgAwACwAIAAxADMALgA5ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABlAHQAcgBvAGwAZQB1AG0AIABiAGEAcwBlAGQAIABnAHIAZQBhAHMAZQBzAFwAIgAsACAAMwA4AC4AOAAsACAAXAAiAGsAbABcACIALAAgADMALgA1ACwAIAAwAC4AMAAsACAAMAAuADAALAAgADMALgA1ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwByAHUAZABlACAAbwBpAGwAIABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgB1AGQAZQAgAG8AaQBsACAAYwBvAG4AZABlAG4AcwBhAHQAZQBzAFwAIgAsACAANAA1AC4AMwAsACAAXAAiAHQAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAANgA5AC4AOAA4ACwAIABcACIATgBFAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGwAaQBxAHUAaQBkAHMAXAAiACwAIAA0ADYALgA1ACwAIABcACIAdABcACIALAAgADYAMQAuADAALAAgADAALgAwADgALAAgADAALgAyACwAIAA2ADEALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB1AHQAbwBtAG8AdABpAHYAZQAgAGcAYQBzAG8AbABpAG4AZQAgAC8AIABwAGUAdAByAG8AbAAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADQALgAyACwAIABcACIAawBMAFwAIgAsACAANgA3AC4ANAAsACAAMAAuADIALAAgADAALgAyACwAIAA2ADcALgA4ADAALAAgADEANwAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AIABnAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADMALgAxACwAIABcACIAawBMAFwAIgAsACAANgA3ACwAIAAwAC4AMgAsACAAMAAuADIALAAgADYANwAuADQAMAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEsAZQByAG8AcwBlAG4AZQAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADcALgA1ACwAIABcACIAawBMAFwAIgAsACAANgA4AC4AOQAsACAAMAAuADAAMQAsACAAMAAuADIALAAgADYAOQAuADEAMQAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgAgAHQAdQByAGIAaQBuAGUAIABmAHUAZQBsACAALwAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAAyACwAIAAwAC4AMgAsACAANgA5AC4AOAAyACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdABpAG4AZwAgAG8AaQBsAFwAIgAsACAAMwA3AC4AMwAsACAAXAAiAGsATABcACIALAAgADYAOQAuADUALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA3ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsATABcACIALAAgADYAOQAuADkALAAgADAALgAxACwAIAAwAC4AMgAsACAANwAwAC4AMgAwACwAIAAxADcALgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAG8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAAXAAiAGsATABcACIALAAgADcAMwAuADYALAAgADAALgAwADQALAAgADAALgAyACwAIAA3ADMALgA4ADQALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAGEAcgBvAG0AYQB0AGkAYwAgAGgAeQBkAHIAbwBjAGEAcgBiAG8AbgBzAFwAIgAsACAAMwA0AC4ANAAsACAAXAAiAGsATABcACIALAAgADYAOQAuADcALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA5ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbAB2AGUAbgB0AHMAOgAgAG0AaQBuAGUAcgBhAGwAIAB0AHUAcgBwAGUAbgB0AGkAbgBlACAAbwByACAAdwBoAGkAdABlACAAcwBwAGkAcgBpAHQAcwBcACIALAAgADMANAAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA3ACwAIAAwAC4AMAAzACwAIAAwAC4AMgAsACAANgA5AC4AOQAzACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABwAGUAdAByAG8AbABlAHUAbQAgAGcAYQBzACAAKABMAFAARwApAFwAIgAsACAAMgA1AC4ANwAsACAAXAAiAGsATABcACIALAAgADYAMAAuADIALAAgADAALgAyACwAIAAwAC4AMgAsACAANgAwAC4ANgAwACwAIAAyADAALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHAAaAB0AGgAYQBcACIALAAgADMAMQAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAA2ADkALgA4ADIALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGMAbwBrAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAdABcACIALAAgADkAMgAuADYALAAgADAALgAwADgALAAgADAALgAyACwAIAA5ADIALgA4ADgALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAZgBpAG4AZQByAHkAIABnAGEAcwAgAGEAbgBkACAAbABpAHEAdQBpAGQAcwBcACIALAAgADQAMgAuADkALAAgAFwAIgB0AFwAIgAsACAANQA0AC4ANwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAANQA0AC4ANwA2ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAGYAaQBuAGUAcgB5ACAAYwBvAGsAZQBcACIALAAgADMANAAuADIALAAgAFwAIgB0AFwAIgAsACAAOQAyAC4ANgAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADkAMgAuADgAOAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAbwB0AGgAZQByACAAdABoAGEAbgAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAzADQALgA0ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOAAsACAAMAAuADAAMgAsACAAMAAuADEALAAgADYAOQAuADkAMgAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA0AC4ANgAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBFAHQAaABhAG4AbwBsACAAZgBvAHIAIAB1AHMAZQAgAGEAcwAgAGEAIABmAHUAZQBsACAAaQBuACAAYQBuACAAaQBuAHQAZQByAG4AYQBsACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAGUAbgBnAGkAbgBlAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGkAbwBmAHUAZQBsAHMAIABvAHQAaABlAHIAIAB0AGgAYQBuACAAdABoAG8AcwBlACAAbQBlAG4AdABpAG8AbgBlAGQAIABpAG4AIAB0AGgAZQAgAGkAdABlAG0AcwAgAGEAYgBvAHYAZQAgAGEAbgBkACAAYgBlAGwAbwB3AFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGEAdgBpAGEAdABpAG8AbgAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADAALgAyADIALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMwAwACwAIABcACIATgBFAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAJwBOAEUAJwAgAHYAYQBsAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAYQBzACAAegBlAHIAbwAgAGYAbwByACAAYwBhAGwAYwB1AGwAYQB0AGkAbwBuAHMALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAVAByAGEAbgBzAHAAbwByAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABUAHIAYQBuAHMAcABvAHIAdABcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMQApACAAYQBuAGQAIABpAG4AZABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAdAByAGEAbgBzAHAAbwByAHQAIABmAHUAZQBsAHMAIABpAG4AIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBxAHUAaQBwAG0AZQBuAHQAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADkAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADYALAAgADEAMAAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAHQAeQBwAGUAXAAiACwAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACgARwBKACAAcABlAHIAIAB1AG4AaQB0ACAAbwBmACAAZgB1AGUAbAApAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB1AG4AaQB0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMATwAyAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMASAA0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAE4AMgBPAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMAbwBtAGIAaQBuAGUAZAAgAGcAYQBzAGUAcwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBHAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAawBsAFwAIgAsACAANgA3AC4ANAAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADYANwAuADYAMgAsACAAMQA3AC4AMgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMAAxACwAIAAwAC4ANQAsACAANwAwAC4ANAAxACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAHAAZQB0AHIAbwBsAGUAdQBtACAAZwBhAHMAIAAoAEwAUABHACkAXAAiACwAIAAyADYALgAyACwAIABcACIAawBsAFwAIgAsACAANgAwAC4AMgAsACAAMAAuADUALAAgADAALgAzACwAIAA2ADEALgAwADAALAAgADIAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEYAdQBlAGwAIABvAGkAbABcACIALAAgADMAOQAuADcALAAgAFwAIgBrAGwAXAAiACwAIAA3ADMALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4ANQAsACAANwA0AC4AMQA4ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBFAHQAaABhAG4AbwBsAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMgAsACAAMAAuADIALAAgADAALgA0ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAQgBpAG8AZABpAGUAcwBlAGwAXAAiACwAIAAzADQALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgA4ACwAIAAxAC4ANwAsACAAMgAuADUALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMAAxACwAIAAwAC4ANQAsACAAMAAuADUAMQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAE8AdABoAGUAcgAgAGIAaQBvAGYAdQBlAGwAcwBcACIALAAgADIAMwAuADQALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADgALAAgADEALgA3ACwAIAAyAC4ANQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAZwBoAHQAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEMAbwBtAHAAcgBlAHMAcwBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADcALgAzACwAIAAwAC4AMwAsACAANQA5AC4AMAAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAaQBnAGgAdAAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBsAFwAIgAsACAANQAxAC4ANAAsACAANwAuADMALAAgADAALgAzACwAIAA1ADkALgAwACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBDAG8AbQBwAHIAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAyAC4AOAAsACAAMAAuADMALAAgADUANAAuADUALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMgA1AC4AMwAsACAAXAAiAGsAbABcACIALAAgADUAMQAuADQALAAgADIALgA4ACwAIAAwAC4AMwAsACAANQA0AC4ANQAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbAAgAC0AIABFAHUAcgBvACAAaQB2ACAAbwByACAAaABpAGcAaABlAHIAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADAANwAsACAAMAAuADQALAAgADcAMAAuADMANwAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbAAgAC0AIABFAHUAcgBvACAAaQBpAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADEALAAgADAALgA0ACwAIAA3ADAALgA0ACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsACAALQAgAEUAdQByAG8AIABpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADkALAAgADAALgAyACwAIAAwAC4ANAAsACAANwAwAC4ANQAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbAAgABMgIABFAHUAcgBvACAAaQB2ACAAbwByACAAaABpAGcAaABlAHIAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAwADcALAAgADAALgA0ACwAIAAwAC4ANAA3ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbAAgABMgIABFAHUAcgBvACAAaQBpAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAxACwAIAAwAC4ANAAsACAAMAAuADUALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsACAAEyAgAEUAdQByAG8AIABpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMgAsACAAMAAuADQALAAgADAALgA2ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAGEAcwBvAGwAaQBuAGUAIABmAG8AcgAgAHUAcwBlACAAYQBzACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGEAaQByAGMAcgBhAGYAdABcACIALAAgADMAMwAuADEALAAgAFwAIgBrAGwAXAAiACwAIAA2ADcALgAwACwAIAAwAC4AMAA2ACwAIAAwAC4ANgAsACAANgA3AC4ANgA2ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB2AGkAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEsAZQByAG8AcwBlAG4AZQAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0AFwAIgAsACAAMwA2AC4AOAAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADYALAAgADAALgAwADEALAAgADAALgA2ACwAIAA3ADAALgAyADEALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABhAHYAaQBhAHQAaQBvAG4AIABrAGUAcgBvAHMAZQBuAGUAXAAiACwAIAAzADYALgA4ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAwADEALAAgADAALgA2ACwAIAAwAC4ANgAxACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAHMAXAAiACwAIABcACIARwBhAHMAbwBsAGkAbgBlAFwAIgAsACAAMwA0AC4AMgAsACAAXAAiAGsATABcACIALAAgADYANwAuADQALAAgADEAMAAuADEALAAgADAALgAzACwAIABcACIAXAAiACwAIAAxADcALgAyACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADIALAAgADAALgA1ACwAIABcACIAXAAiACwAIAAxADcALgAzACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABzAFwAIgAsACAAXAAiAEYAdQBlAGwAIABPAGkAbABcACIALAAgADMAOQAuADcALAAgAFwAIgBrAEwAXAAiACwAIAA3ADMALgA2ACwAIAAwAC4AMgAsACAAMAAuADUALAAgAFwAIgBcACIALAAgADEAOAAuADAALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE8AZgBmAC0AcgBvAGEAZAAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAgAGEAbgBkACAAZgBvAHIAZQBzAHQAcgB5ACAAZQBxAHUAaQBwAG0AZQBuAHQAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMwAsACAAMAAuADUALAAgAFwAIgBcACIALAAgADEANwAuADMALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgACcATgBFACcAIAB2AGEAbAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAGEAcwAgAHoAZQByAG8AIABmAG8AcgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABPAGYAZgAtAHIAYQBkACAAZQBxAHUAaQBwAG0AZQBuAHQAIABhAG4AZAAgAHYAZQBzAHMAZQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABhAG4AZAAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAE8AZgBmAC0AcgBvAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADEAKQAgAGEAbgBkACAAaQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAzACkAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwAgAGkAbgAgAG8AZgBmAC0AcgBvAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAA3ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBwAG8AcgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIARgB1AGUAbAAgAHQAeQBwAGUAIABxAFwAIgAsACAAXAAiAEUAQwBUAHIAYQBuAHMALABxACAAKABHAEoALwBrAEwAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAAQwBPADIAIABFAEYAVAByAGEAbgAsADEALAB0AHEAZwAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEMASAA0ACAARQBGAFQAcgBhAG4ALAAxACwAdABnAGcAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABOADIATwAgAEUARgBUAHIAYQBuACwAMQAsAHQAZwBnACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBGAFQAcgBhAG4AcwAsADMALABxACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABcACIALAAgAFwAIgBQAGUAdAByAG8AbABcACIALAAgADMANAAuADIALAAgADYANwAuADQALAAgADEAMAAuADEALAAgADAALgAzACwAIAAxADcALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIARABpAGUAcwBlAGwAXAAiACwAIAAzADgALgA2ACwAIAA2ADkALgA5ACwAIAAwAC4AMgAsACAAMAAuADUALAAgADEANwAuADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABcACIALAAgAFwAIgBGAHUAZQBsACAATwBpAGwAXAAiACwAIAAzADkALgA3ACwAIAA3ADMALgA2ACwAIAAwAC4AMgAsACAAMAAuADUALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBPAGYAZgAtAHIAbwBhAGQAIABBAGcAcgBpAGMAdQBsAHQAdQByAGUAIABhAG4AZAAgAGYAbwByAGUAcwB0AHIAeQAgAGUAcQB1AGkAcABtAGUAbgB0AFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAANgA5AC4AOQAsACAAMAAuADMALAAgADAALgA1ACwAIAAxADcALgAzAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARgB1AGUAbABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAEYAdQBlAGwAXwBHAGUAdABUAHIAYQBuAHMAcABvAHIAdABGAHUAZQBsAFMAdAByAGkAbgBnAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsAFwAbgAgACAAIAAgAEwARQBGAFQAKABDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAIABcACIALABDAGUAbABsACkAIAAtADEAKQBcAG4AKQA7AFwAbgBcAG4ARgB1AGUAbABfAEcAZQB0AFMAdABhAHQAaQBvAG4AYQByAHkARgB1AGUAbABTAHQAcgBpAG4AZwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALABcAG4AIAAgACAAIABSAEkARwBIAFQAKABDAGUAbABsACwAIABMAEUATgAoAEMAZQBsAGwAKQAgAC0AIABGAEkATgBEACgAXAAiACwAIABcACIALAAgAEMAZQBsAGwAKQAgAC0AIAAxACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBUAG8AdABhAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAFwAbgA9ACAATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABGAHUAZQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgBBAHIAcgBhAHkALAAgAEYAdQBlAGwAVQBzAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFUAcwBlACwAIABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFQAeQBwAGUALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAUwBVAE0AKABcAG4AIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAEYAdQBlAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACAAPQAgAEYAdQBlAGwAVAB5AHAAZQApACAAKgAgAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFUAcwBlAEEAcgByAGEAeQAgAD0AIABGAHUAZQBsAFUAcwBlACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQAsAFwAbgAgACAAIAAgADAAXABuACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AOAA6ACAARgB1AGUAbAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADgALgAxACAARgB1AGUAbAAgAFUAcwBlACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0ACAAZgB1AGUAbABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRACwAIABFAEMALAAgAEUARgAsAFwAbgAgACAAIAAgACgAUQAgACoAIABFAEMAIAAqACAARQBGACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAYwBvAG0AYgB1AHMAdABlAGQAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAAawBMAFwAbgBFAEMAIAA6ACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAOgAgAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBUAHIAYQBuAHMAdABxACwAIABFAEMAXwBUAHIAYQBuAHMAcQAsACAARQBGAF8AVAByAGEAbgBzADEAdABxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFQAcgBhAG4AcwB0AHEALAAgAEUAQwBfAFQAcgBhAG4AcwBxACwAIABFAEYAXwBUAHIAYQBuAHMAMQB0AHEAZwApAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsAVAByAGEAbgBzACwAdABxAH0AXABcAHQAaQBtAGUAcwAgAEUAQwBfAHsAVAByAGEAbgBzACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFQAcgBhAG4AcwAsADEALAB0AHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAFQAcgBhAG4AcwB0AHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIABjAG8AbQBiAHUAcwB0AGUAZAAgAGYAbwByACAAdAByAGEAbgBzAHAAbwByAHQAIABlAG4AZQByAGcAeQAgAHAAdQByAHAAbwBzAGUAcwBcACIALAAgAFwAIgBWAGEAcgBpAGUAcwAgAGIAYQBzAGUAZAAgAG8AbgAgAGYAdQBlAGwAIAB0AHkAcABlADoAIABrAEwALAAgAG0AMwAsACAARwBKAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAF8AVAByAGEAbgBzAHEAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AVAByAGEAbgBzADEAdABxAGcAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBcACIALAAgAFwAIgBGAHUAZQBsACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBcACIALAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwBcAG4AUQAgADoAIABBAG0AbwB1AG4AdAAgAG8AZgAgAGYAdQBlAGwAIAB0AHkAcABlACAAcQAgAHUAcwBlAGQAIABmAG8AcgAgAHMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBwAGUAcgBhAHQAaQBvAG4AcwAgADoAIABrAEwAXABuAEUAQwAgADoAIABFAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAEcASgAvAGsATABcAG4ARQBGACAAOgAgAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIAA6ACAAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AUwBDAHEALAAgAEUAQwBfAFMAQwBxACwAIABFAEYAXwBTAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFMAQwBxACwAIABFAEMAXwBTAEMAcQAsACAARQBGAF8AUwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAbwByACAAZQBhAGMAaAAgAEcASABHACAAZgByAG8AbQAgAHQAaABlACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdAAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AcQBcAFwAbABlAGYAdAAoAFEAXwB7AFMAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBDAF8AewBTAEMALABxAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUwBDACwAMQAsAHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AUwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAFMAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AUwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBDAFwAIgAsACAAXAAiAFMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADIAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBcAG4ARQBtAGkAcwBzAGkAbwBuAHMAIABmAG8AcgAgAGUAYQBjAGgAIABHAEgARwAgAGYAcgBvAG0AIABnAGUAbgBlAHIAaQBjACAAZgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIAB3AGgAZQByAGUAIAB0AGgAZQAgAHUAcwBhAGcAZQAgAGkAcwAgAG4AbwB0ACAAawBuAG8AdwBuAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAdQBzAGUAZAAgAGYAbwByACAAZwBlAG4AZQByAGkAYwAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAGsATABcAG4ARQBDACAAOgAgAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgADoAIABrAGcAIABDAE8AMgBlACAALwAgAEcASgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8ARwBDAHEALAAgAEUAQwBfAEcAQwBxACwAIABFAEYAXwBHAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAEcAQwBxACwAIABFAEMAXwBHAEMAcQAsACAARQBGAF8ARwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAG8AcgAgAGUAYQBjAGgAIABHAEgARwAgAGYAcgBvAG0AIAB0AGgAZQAgAGcAZQBuAGUAcgBpAGMAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVQBzAGUAcwAgAFYARQBFAFIARwAgADIAMAAyADYAOgAgADgALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApACwAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQAgAGEAbgBkACAAZQB2AGUAcgBhAGcAZQBzACAAdABoAGUAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGEAbgBkACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAZwBlAG4AZQByAGkAYwAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzACAAYQBuAGQAIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsARwBDACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEMAXwB7AEcAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBHAEMALAAxACwAcQBnAH0AXABcAHIAaQBnAGgAdAApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8ARwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAEcAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8ARwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwBlAG4AZQByAGkAYwAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBDAFwAIgAsACAAXAAiAEcAZQBuAGUAcgBpAGMAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAVABoAGkAcwAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAgAHUAcwBlAHMAIABhAHYAZQByAGEAZwBlAHMAIABvAGYAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGEAbgBkACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAdwBoAGUAcgBlACAAdABoAGUAIAB1AHMAYQBnAGUAIABpAHMAIABuAG8AdAAgAGsAbgBvAHcAbgAuAFwAIgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGEAdABhACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AE8AZgBmAFIAbwBhAGQAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEYAdQBlAGwAXwBHAGUAdABUAHIAYQBuAHMAcABvAHIAdABGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8ARwBlAHQAUwB0AGEAdABpAG8AbgBhAHIAeQBGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8AVABvAHQAYQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBVAG4AaQB0ACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVQBuAGkAdAAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -22817,7 +22581,20 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzACAAaQBuAGMAbAB1AGQAaQBuAGcAIABsAGkAcQB1AGUAZgBpAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgACAAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA1AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAANwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAHUAZQBsACAAYwBvAG0AYgB1AHMAdABlAGQAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABDAG8AbgB0AGUAbgB0ACAARgBhAGMAdABvAHIAIAAoAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwAKQBcACIALAAgAFwAIgBGAHUAZQBsACAAdQBuAGkAdABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAE8AMgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAEgANABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOADIATwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAG8AbQBiAGkAbgBlAGQAIABnAGEAcwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIAAwAC4AMAAzADcANwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADAALgAyACwAIAAwAC4AMAAzACwAIAA1ADEALgA2ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AYQBsACAAbQBpAG4AZQAgAHcAYQBzAHQAZQAgAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4AOQAsACAANAAuADYALAAgADAALgAzACwAIAA1ADYALgA4ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcAByAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAoAHIAZQB2AGUAcgB0AGkAbgBnACAAdABvACAAcwB0AGEAbgBkAGEAcgBkACAAYwBvAG4AZABpAHQAaQBvAG4AcwApAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVQBuAHAAcgBvAGMAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAA2ADIAOQAsACAAXAAiAG0AMwBcACIALAAgADUANgAuADUALAAgADAALgAwADMALAAgADAALgAwADMALAAgADUANgAuADUANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBrAGUAIABvAHYAZQBuACAAZwBhAHMAXAAiACwAIAAwAC4AMAAxADgAMQAsACAAXAAiAG0AMwBcACIALAAgADMANwAuADAALAAgADAALgAwADMALAAgADAALgAwADUALAAgADMANwAuADAAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAbABhAHMAdAAgAGYAdQByAG4AYQBjAGUAIABnAGEAcwBcACIALAAgADAALgAwADAANAAwACwAIABcACIAbQAzAFwAIgAsACAAMgAzADQALgAwACwAIAAwAC4AMAAzACwAIAAwAC4AMAAyACwAIAAyADMANAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwBcACIALAAgADAALgAwADMAOQAwACwAIABcACIAbQAzAFwAIgAsACAANgAwAC4AMgAsACAAMAAuADAANAAsACAAMAAuADAAMwAsACAANgAwAC4AMgA3ADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBMAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAGUAbwB1AHMAIABmAG8AcwBzAGkAbAAgAGYAdQBlAGwAcwAgAG8AdABoAGUAcgAgAHQAaABhAG4AIAB0AGgAbwBzAGUAIABtAGUAbgB0AGkAbwBuAGUAZAAgAGkAbgAgAHQAaABlACAAaQB0AGUAbQBzACAAYQBiAG8AdgBlAFwAIgAsACAAMAAuADAAMwA5ADAALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsACAAYgBpAG8AZwBhAHMAIAB0AGgAYQB0ACAAaQBzACAAYwBhAHAAdAB1AHIAZQBkACAAZgBvAHIAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAKABtAGUAdABoAGEAbgBlACAAbwBuAGwAeQApAFwAIgAsACAAMAAuADAAMwA3ADcALAAgAFwAIgBtADMAXAAiACwAIAAwAC4AMAAsACAANgAuADQALAAgADAALgAwADMALAAgADYALgA0ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgACgAbQBlAHQAaABhAG4AZQAgAG8AbgBsAHkAKQBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADYALgA0ACwAIAAwAC4AMAAzACwAIAA2AC4ANAAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAsACAAbwB0AGgAZQByACAAdABoAGEAbgAgAHQAaABvAHMAZQAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAwAC4AMAAzADcAMAAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAA2AC4ANAAsACAAMAAuADAAMwAsACAANgAuADQAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAG0AZQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAAMAAuADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAeQBkAHIAbwBnAGUAbgBcACIALAAgADAALgAwADEAMgAyACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADAALgAwACwAIAAwAC4ANQAsACAAMAAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdAB1AHIAYQBsACAAZwBhAHMAIABkAGkAcwB0AHIAaQBiAHUAdABlAGQAIABpAG4AIABhACAAcABpAHAAZQBsAGkAbgBlACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAXAAiACwAIAAxACwAIABcACIARwBKAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzAFwAIgAsACAAMQAsACAAXAAiAEcASgBcACIALAAgADYAMAAuADIALAAgADAALgAwADQALAAgADAALgAwADMALAAgADYAMAAuADIANwBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgACcATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzACcAIABhAG4AZAAgACcAVABvAHcAbgAgAGcAYQBzACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAJwAgAHcAZQByAGUAIABhAGQAZABlAGQALAAgAGUAYQBjAGgAIAB3AGkAdABoACAAYQBuACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABvAGYAIAAxACAARwBKACAAcABlAHIAIAB1AG4AaQB0ACAAbwBmACAAZgB1AGUAbAAuACAAVABoAGkAcwAgAGkAcwAgAGYAbwByACAAdQBzAGUAcgBzACAAdwBoAG8AIABoAGEAdgBlACAAZgB1AGUAbAAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGQAYQB0AGEAIABpAG4AIABHAEoAIAByAGEAdABoAGUAcgAgAHQAaABhAG4AIABtADMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGcAYQBzAGUAbwB1AHMAIABmAHUAZQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBGAHUAZQBsACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGcAYQBzAGUAbwB1AHMAIABmAHUAZQBsAHMAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMALgBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADYAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAB0AGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgAGYAbwByACAATgBhAHQAdQByAGEAbAAgAEcAYQBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATQBlAHQAcgBvAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgBzACAAZgBvAHIAIABOAGEAdAB1AHIAYQBsACAARwBhAHMAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOAG8AbgAgAC0AIABNAGUAdAByAG8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIAAxADMALgAxACwAIAAxADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBDAFQAXAAiACwAIAAxADMALgAxACwAIAAxADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAANAAuADAALAAgADQALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgADgALgA4ACwAIAA3AC4AOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAMQAwAC4ANwAsACAAMQAwAC4ANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADQALgAxACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgADQALgAwACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAANAAuADEALAAgADQALgAwAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATgBTAFcAIABhAG4AZAAgAEEAQwBUACAAcwBwAGwAaQB0ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAHIAbwB3AHMALgAgACcAQwAnACAAVgBhAGwAdQBlAHMAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAGEAbgBkACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAByAGUAcABsAGEAYwBlAGQAIAB3AGkAdABoACAAdABoAG8AcwBlACAAZgBvAHIAIABWAGkAYwB0AG8AcgBpAGEAIABhAG4AZAAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAHIAZQBzAHAAZQBjAHQAaQB2AGUAbAB5AC4AIAAoAFMAZQBlACAAYQBwAHAAZQBuAGQAaQBjAGUAcwApAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEEAcwAgAFMAYwBvAHAAZQAgADMAIABmAGEAYwB0AG8AcgBzACAAYQByAGUAIABjAGEAbABjAHUAbABhAHQAZQBkACAAYQB0ACAAdABoAGUAIABwAG8AaQBuAHQAIAB3AGgAZQByAGUAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIABpAHMAIABkAGUAbABpAHYAZQByAGUAZAAgAHQAbwAgAGUAbgBkACAAdQBzAGUAcgBzACwAIABpAHQAIABpAHMAIABuAGUAYwBlAHMAcwBhAHIAeQAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAYQB0ACAAZQBhAGMAaAAgAG8AZgAgAHQAaABlACAAbABvAGEAZAAgAGMAZQBuAHQAcgBlAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBHAGEAcwAgAHIAZQBhAGMAaABlAHMAIABlAG4AZAAgAHUAcwBlAHIAcwAgAGUAaQB0AGgAZQByACAAZgByAG8AbQAgAHQAaABlACAAbQBlAHQAcgBvACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABuAGUAdAB3AG8AcgBrAHMAIABvAHIAIABkAGkAcgBlAGMAdAAgAGYAcgBvAG0AIAB0AGgAZQAgAGgAaQBnAGgAIAAtACAAcAByAGUAcwBzAHUAcgBlACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABwAGkAcABlAGwAaQBuAGUAcwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAEgAbwB1AHMAZQBoAG8AbABkAHMAIABhAG4AZAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB1AHMAZQByAHMAIAB0AGUAbgBkACAAdABvACAAYgBlACAAcwBlAHIAdgBlAGQAIABiAHkAIAB0AGgAZQAgAGYAbwByAG0AZQByACwAIABhAG4AZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAGcAZQBuAGUAcgBhAHQAbwByAHMAIABhAG4AZAAgAGwAYQByAGcAZQAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIABwAGwAYQBuAHQAcwAgAGYAcgBvAG0AIAB0AGgAZQAgAGwAYQB0AHQAZQByAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBNAGUAdAByAG8AIABpAHMAIABkAGUAZgBpAG4AZQBkACAAYQBzACAAbABvAGMAYQB0AGUAZAAgAG8AbgAgAG8AcgAgAGUAYQBzAHQAIABvAGYAIAB0AGgAZQAgAGQAaQB2AGkAZABpAG4AZwAgAHIAYQBuAGcAZQAgAGkAbgAgAE4AUwBXACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAEMAYQBuAGIAZQByAHIAYQAgAGEAbgBkACAAUQB1AGUAYQBuAGIAZQB5AGEAbgAsACAATQBlAGwAYgBvAHUAcgBuAGUALAAgAEIAcgBpAHMAYgBhAG4AZQAsACAAQQBkAGUAbABhAGkAZABlACAAbwByACAAUABlAHIAdABoAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIATwB0AGgAZQByAHcAaQBzAGUALAAgAHQAaABlACAAbgBvAG4AIAAtACAAbQBlAHQAcgBvACAAZgBhAGMAdABvAHIAIABzAGgAbwB1AGwAZAAgAGIAZQAgAHUAcwBlAGQALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEYAYQBjAHQAbwByAHMAIABhAHIAZQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAGEAbABsACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAHcAaABpAGMAaAAgAG0AYQB5ACAAaQBuAGMAbAB1AGQAZQAgAGMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACwAIABcACIAVABhAGIAbABlACAANgAgAGkAcwAgAG4AbwB0ACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHQAbwAgAGUAdABoAGEAbgBlAC4AIABTAGUAZQAgAFQAYQBiAGwAZQAgADcAIABJAG4AZABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAZQB0AGgAYQBuAGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEMAIAA9ACAAQwBvAG4AZgBpAGQAZQBuAHQAaQBhAGwALgAgAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABUAGEAcwBtAGEAbgBpAGEAIABhAG4AZAAgAHQAaABlACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIABhAHIAZQAgAG4AbwB0ACAAYQB2AGEAaQBsAGEAYgBsAGUAIABkAHUAZQAgAHQAbwAgAGMAbwBuAGYAaQBkAGUAbgB0AGkAYQBsAGkAdAB5ACAAYwBvAG4AcwB0AHIAYQBpAG4AdABzACAAdABoAGEAdAAgAGEAcgBpAHMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBmAHIAbwBtACAAdABoAGUAIAB1AHMAZQAgAG8AZgAgAGEAIABsAGkAbQBpAHQAZQBkACAAbgB1AG0AYgBlAHIAIABvAGYAIABOAEcARQBSACAAZABhAHQAYQAgAGkAbgBwAHUAdABzAC4AIABJAHQAIABpAHMAIABzAHUAZwBnAGUAcwB0AGUAZAAgAHQAaABhAHQAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAHQAaABlACAAdQBzAGUAIABvAGYAIAB0AGgAZQAgAFYAaQBjAHQAbwByAGkAYQBuACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGkAcwAgAGEAcABwAHIAbwBwAHIAaQBhAHQAZQAsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAHcAaABpAGwAZQAgAGYAbwByACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAB0AGgAZQAgAHUAcwBlACAAbwBmACAAdABoAGUAIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABpAHMAIABhAHAAcAByAG8AcAByAGkAYQB0AGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZABvACAAbgBvAHQAIABpAG4AYwBsAHUAZABlACAAZgB1AGcAaQB0AGkAdgBlACAAZQBtAGkAcwBzAGkAbwBuACAAbABlAGEAawBhAGcAZQAgAGYAcgBvAG0AIABsAG8AdwAgAHAAcgBlAHMAcwB1AHIAZQAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGkAbwBuACAAcABpAHAAZQBsAGkAbgBlACAAbgBlAHQAdwBvAHIAawBzACAAdwBoAGkAbABlACAAdABoAG8AcwBlACAAZgByAG8AbQAgAGgAaQBnAGgAIABwAHIAZQBzAHMAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAZwBhAHMAIABuAGUAdAB3AG8AcgBrAHMAIABhAHIAZQAgAGMAbwBuAHMAaQBkAGUAcgBlAGQAIABuAGUAZwBsAGkAZwBpAGIAbABlAC4AXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABTAHQAYQB0AGkAbwBuAGEAcgB5ACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAYQBuAGQAIABpAG4AZABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMALAAgAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBlAHIAdABhAGkAbgAgAHAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMALgBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA4AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADUALAAgADgALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACAAKABHAEoAIABwAGUAcgAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsACkAXAAiACwAIABcACIARgB1AGUAbAAgAHUAbgBpAHQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBPADIAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBIADQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgAyAE8AXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBvAG0AYgBpAG4AZQBkACAAZwBhAHMAZQBzAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsAHMAIAAoAG8AdABoAGUAcgAgAHQAaABhAG4AIABwAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsACAAdQBzAGUAZAAgAGEAcwAgAGYAdQBlAGwAKQAsACAAZQAuAGcALgAgAGwAdQBiAHIAaQBjAGEAbgB0AHMAXAAiACwAIAAzADgALgA4ACwAIABcACIAawBsAFwAIgAsACAAMQAzAC4AOQAsACAAMAAuADAALAAgADAALgAwACwAIAAxADMALgA5ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABlAHQAcgBvAGwAZQB1AG0AIABiAGEAcwBlAGQAIABnAHIAZQBhAHMAZQBzAFwAIgAsACAAMwA4AC4AOAAsACAAXAAiAGsAbABcACIALAAgADMALgA1ACwAIAAwAC4AMAAsACAAMAAuADAALAAgADMALgA1ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwByAHUAZABlACAAbwBpAGwAIABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgB1AGQAZQAgAG8AaQBsACAAYwBvAG4AZABlAG4AcwBhAHQAZQBzAFwAIgAsACAANAA1AC4AMwAsACAAXAAiAHQAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAANgA5AC4AOAA4ACwAIABcACIATgBFAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGwAaQBxAHUAaQBkAHMAXAAiACwAIAA0ADYALgA1ACwAIABcACIAdABcACIALAAgADYAMQAuADAALAAgADAALgAwADgALAAgADAALgAyACwAIAA2ADEALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB1AHQAbwBtAG8AdABpAHYAZQAgAGcAYQBzAG8AbABpAG4AZQAgAC8AIABwAGUAdAByAG8AbAAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADQALgAyACwAIABcACIAawBMAFwAIgAsACAANgA3AC4ANAAsACAAMAAuADIALAAgADAALgAyACwAIAA2ADcALgA4ADAALAAgADEANwAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AIABnAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADMALgAxACwAIABcACIAawBMAFwAIgAsACAANgA3ACwAIAAwAC4AMgAsACAAMAAuADIALAAgADYANwAuADQAMAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEsAZQByAG8AcwBlAG4AZQAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADcALgA1ACwAIABcACIAawBMAFwAIgAsACAANgA4AC4AOQAsACAAMAAuADAAMQAsACAAMAAuADIALAAgADYAOQAuADEAMQAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgAgAHQAdQByAGIAaQBuAGUAIABmAHUAZQBsACAALwAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAAyACwAIAAwAC4AMgAsACAANgA5AC4AOAAyACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdABpAG4AZwAgAG8AaQBsAFwAIgAsACAAMwA3AC4AMwAsACAAXAAiAGsATABcACIALAAgADYAOQAuADUALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA3ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsATABcACIALAAgADYAOQAuADkALAAgADAALgAxACwAIAAwAC4AMgAsACAANwAwAC4AMgAwACwAIAAxADcALgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAG8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAAXAAiAGsATABcACIALAAgADcAMwAuADYALAAgADAALgAwADQALAAgADAALgAyACwAIAA3ADMALgA4ADQALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAGEAcgBvAG0AYQB0AGkAYwAgAGgAeQBkAHIAbwBjAGEAcgBiAG8AbgBzAFwAIgAsACAAMwA0AC4ANAAsACAAXAAiAGsATABcACIALAAgADYAOQAuADcALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA5ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbAB2AGUAbgB0AHMAOgAgAG0AaQBuAGUAcgBhAGwAIAB0AHUAcgBwAGUAbgB0AGkAbgBlACAAbwByACAAdwBoAGkAdABlACAAcwBwAGkAcgBpAHQAcwBcACIALAAgADMANAAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA3ACwAIAAwAC4AMAAzACwAIAAwAC4AMgAsACAANgA5AC4AOQAzACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABwAGUAdAByAG8AbABlAHUAbQAgAGcAYQBzACAAKABMAFAARwApAFwAIgAsACAAMgA1AC4ANwAsACAAXAAiAGsATABcACIALAAgADYAMAAuADIALAAgADAALgAyACwAIAAwAC4AMgAsACAANgAwAC4ANgAwACwAIAAyADAALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHAAaAB0AGgAYQBcACIALAAgADMAMQAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAA2ADkALgA4ADIALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGMAbwBrAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAdABcACIALAAgADkAMgAuADYALAAgADAALgAwADgALAAgADAALgAyACwAIAA5ADIALgA4ADgALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAZgBpAG4AZQByAHkAIABnAGEAcwAgAGEAbgBkACAAbABpAHEAdQBpAGQAcwBcACIALAAgADQAMgAuADkALAAgAFwAIgB0AFwAIgAsACAANQA0AC4ANwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAANQA0AC4ANwA2ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAGYAaQBuAGUAcgB5ACAAYwBvAGsAZQBcACIALAAgADMANAAuADIALAAgAFwAIgB0AFwAIgAsACAAOQAyAC4ANgAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADkAMgAuADgAOAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAbwB0AGgAZQByACAAdABoAGEAbgAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAzADQALgA0ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOAAsACAAMAAuADAAMgAsACAAMAAuADEALAAgADYAOQAuADkAMgAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA0AC4ANgAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBFAHQAaABhAG4AbwBsACAAZgBvAHIAIAB1AHMAZQAgAGEAcwAgAGEAIABmAHUAZQBsACAAaQBuACAAYQBuACAAaQBuAHQAZQByAG4AYQBsACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAGUAbgBnAGkAbgBlAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGkAbwBmAHUAZQBsAHMAIABvAHQAaABlAHIAIAB0AGgAYQBuACAAdABoAG8AcwBlACAAbQBlAG4AdABpAG8AbgBlAGQAIABpAG4AIAB0AGgAZQAgAGkAdABlAG0AcwAgAGEAYgBvAHYAZQAgAGEAbgBkACAAYgBlAGwAbwB3AFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGEAdgBpAGEAdABpAG8AbgAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADAALgAyADIALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMwAwACwAIABcACIATgBFAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAJwBOAEUAJwAgAHYAYQBsAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAYQBzACAAegBlAHIAbwAgAGYAbwByACAAYwBhAGwAYwB1AGwAYQB0AGkAbwBuAHMALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAVAByAGEAbgBzAHAAbwByAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABUAHIAYQBuAHMAcABvAHIAdABcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMQApACAAYQBuAGQAIABpAG4AZABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAdAByAGEAbgBzAHAAbwByAHQAIABmAHUAZQBsAHMAIABpAG4AIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBxAHUAaQBwAG0AZQBuAHQAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADkAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADYALAAgADEAMAAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAHQAeQBwAGUAXAAiACwAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACgARwBKACAAcABlAHIAIAB1AG4AaQB0ACAAbwBmACAAZgB1AGUAbAApAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB1AG4AaQB0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMATwAyAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMASAA0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAE4AMgBPAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMAbwBtAGIAaQBuAGUAZAAgAGcAYQBzAGUAcwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBHAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAawBsAFwAIgAsACAANgA3AC4ANAAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADYANwAuADYAMgAsACAAMQA3AC4AMgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMAAxACwAIAAwAC4ANQAsACAANwAwAC4ANAAxACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAHAAZQB0AHIAbwBsAGUAdQBtACAAZwBhAHMAIAAoAEwAUABHACkAXAAiACwAIAAyADYALgAyACwAIABcACIAawBsAFwAIgAsACAANgAwAC4AMgAsACAAMAAuADUALAAgADAALgAzACwAIAA2ADEALgAwADAALAAgADIAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEYAdQBlAGwAIABvAGkAbABcACIALAAgADMAOQAuADcALAAgAFwAIgBrAGwAXAAiACwAIAA3ADMALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4ANQAsACAANwA0AC4AMQA4ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBFAHQAaABhAG4AbwBsAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMgAsACAAMAAuADIALAAgADAALgA0ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAQgBpAG8AZABpAGUAcwBlAGwAXAAiACwAIAAzADQALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgA4ACwAIAAxAC4ANwAsACAAMgAuADUALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMAAxACwAIAAwAC4ANQAsACAAMAAuADUAMQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAE8AdABoAGUAcgAgAGIAaQBvAGYAdQBlAGwAcwBcACIALAAgADIAMwAuADQALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADgALAAgADEALgA3ACwAIAAyAC4ANQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAZwBoAHQAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEMAbwBtAHAAcgBlAHMAcwBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADcALgAzACwAIAAwAC4AMwAsACAANQA5AC4AMAAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAaQBnAGgAdAAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBsAFwAIgAsACAANQAxAC4ANAAsACAANwAuADMALAAgADAALgAzACwAIAA1ADkALgAwACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBDAG8AbQBwAHIAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAyAC4AOAAsACAAMAAuADMALAAgADUANAAuADUALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMgA1AC4AMwAsACAAXAAiAGsAbABcACIALAAgADUAMQAuADQALAAgADIALgA4ACwAIAAwAC4AMwAsACAANQA0AC4ANQAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbAAgAC0AIABFAHUAcgBvACAAaQB2ACAAbwByACAAaABpAGcAaABlAHIAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADAANwAsACAAMAAuADQALAAgADcAMAAuADMANwAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbAAgAC0AIABFAHUAcgBvACAAaQBpAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADEALAAgADAALgA0ACwAIAA3ADAALgA0ACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsACAALQAgAEUAdQByAG8AIABpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADkALAAgADAALgAyACwAIAAwAC4ANAAsACAANwAwAC4ANQAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbAAgABMgIABFAHUAcgBvACAAaQB2ACAAbwByACAAaABpAGcAaABlAHIAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAwADcALAAgADAALgA0ACwAIAAwAC4ANAA3ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbAAgABMgIABFAHUAcgBvACAAaQBpAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAxACwAIAAwAC4ANAAsACAAMAAuADUALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsACAAEyAgAEUAdQByAG8AIABpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMgAsACAAMAAuADQALAAgADAALgA2ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgBcACIALAAgAFwAIgBHAGEAcwBvAGwAaQBuAGUAIABmAG8AcgAgAHUAcwBlACAAYQBzACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGEAaQByAGMAcgBhAGYAdABcACIALAAgADMAMwAuADEALAAgAFwAIgBrAGwAXAAiACwAIAA2ADcALgAwACwAIAAwAC4AMAA2ACwAIAAwAC4ANgAsACAANgA3AC4ANgA2ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB2AGkAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEsAZQByAG8AcwBlAG4AZQAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0AFwAIgAsACAAMwA2AC4AOAAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADYALAAgADAALgAwADEALAAgADAALgA2ACwAIAA3ADAALgAyADEALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABhAHYAaQBhAHQAaQBvAG4AIABrAGUAcgBvAHMAZQBuAGUAXAAiACwAIAAzADYALgA4ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAwADEALAAgADAALgA2ACwAIAAwAC4ANgAxACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAHMAXAAiACwAIABcACIARwBhAHMAbwBsAGkAbgBlAFwAIgAsACAAMwA0AC4AMgAsACAAXAAiAGsATABcACIALAAgADYANwAuADQALAAgADEAMAAuADEALAAgADAALgAzACwAIABcACIAXAAiACwAIAAxADcALgAyACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADIALAAgADAALgA1ACwAIABcACIAXAAiACwAIAAxADcALgAzACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABzAFwAIgAsACAAXAAiAEYAdQBlAGwAIABPAGkAbABcACIALAAgADMAOQAuADcALAAgAFwAIgBrAEwAXAAiACwAIAA3ADMALgA2ACwAIAAwAC4AMgAsACAAMAAuADUALAAgAFwAIgBcACIALAAgADEAOAAuADAALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE8AZgBmAC0AcgBvAGEAZAAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAgAGEAbgBkACAAZgBvAHIAZQBzAHQAcgB5ACAAZQBxAHUAaQBwAG0AZQBuAHQAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMwAsACAAMAAuADUALAAgAFwAIgBcACIALAAgADEANwAuADMALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgACcATgBFACcAIAB2AGEAbAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAGEAcwAgAHoAZQByAG8AIABmAG8AcgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABPAGYAZgAtAHIAYQBkACAAZQBxAHUAaQBwAG0AZQBuAHQAIABhAG4AZAAgAHYAZQBzAHMAZQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABhAG4AZAAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAE8AZgBmAC0AcgBvAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADEAKQAgAGEAbgBkACAAaQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAzACkAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwAgAGkAbgAgAG8AZgBmAC0AcgBvAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAA3ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBwAG8AcgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIARgB1AGUAbAAgAHQAeQBwAGUAIABxAFwAIgAsACAAXAAiAEUAQwBUAHIAYQBuAHMALABxACAAKABHAEoALwBrAEwAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAAQwBPADIAIABFAEYAVAByAGEAbgAsADEALAB0AHEAZwAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEMASAA0ACAARQBGAFQAcgBhAG4ALAAxACwAdABnAGcAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABOADIATwAgAEUARgBUAHIAYQBuACwAMQAsAHQAZwBnACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBGAFQAcgBhAG4AcwAsADMALABxACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABcACIALAAgAFwAIgBQAGUAdAByAG8AbABcACIALAAgADMANAAuADIALAAgADYANwAuADQALAAgADEAMAAuADEALAAgADAALgAzACwAIAAxADcALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIARABpAGUAcwBlAGwAXAAiACwAIAAzADgALgA2ACwAIAA2ADkALgA5ACwAIAAwAC4AMgAsACAAMAAuADUALAAgADEANwAuADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABcACIALAAgAFwAIgBGAHUAZQBsACAATwBpAGwAXAAiACwAIAAzADkALgA3ACwAIAA3ADMALgA2ACwAIAAwAC4AMgAsACAAMAAuADUALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBPAGYAZgAtAHIAbwBhAGQAIABBAGcAcgBpAGMAdQBsAHQAdQByAGUAIABhAG4AZAAgAGYAbwByAGUAcwB0AHIAeQAgAGUAcQB1AGkAcABtAGUAbgB0AFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAANgA5AC4AOQAsACAAMAAuADMALAAgADAALgA1ACwAIAAxADcALgAzAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARgB1AGUAbABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAEYAdQBlAGwAXwBHAGUAdABUAHIAYQBuAHMAcABvAHIAdABGAHUAZQBsAFMAdAByAGkAbgBnAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsAFwAbgAgACAAIAAgAEwARQBGAFQAKABDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAIABcACIALABDAGUAbABsACkAIAAtADEAKQBcAG4AKQA7AFwAbgBcAG4ARgB1AGUAbABfAEcAZQB0AFMAdABhAHQAaQBvAG4AYQByAHkARgB1AGUAbABTAHQAcgBpAG4AZwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALABcAG4AIAAgACAAIABSAEkARwBIAFQAKABDAGUAbABsACwAIABMAEUATgAoAEMAZQBsAGwAKQAgAC0AIABGAEkATgBEACgAXAAiACwAIABcACIALAAgAEMAZQBsAGwAKQAgAC0AIAAxACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBUAG8AdABhAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAFwAbgA9ACAATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABGAHUAZQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgBBAHIAcgBhAHkALAAgAEYAdQBlAGwAVQBzAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFUAcwBlACwAIABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFQAeQBwAGUALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAUwBVAE0AKABcAG4AIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAEYAdQBlAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACAAPQAgAEYAdQBlAGwAVAB5AHAAZQApACAAKgAgAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFUAcwBlAEEAcgByAGEAeQAgAD0AIABGAHUAZQBsAFUAcwBlACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQAsAFwAbgAgACAAIAAgADAAXABuACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AOAA6ACAARgB1AGUAbAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADgALgAxACAARgB1AGUAbAAgAFUAcwBlACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0ACAAZgB1AGUAbABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRACwAIABFAEMALAAgAEUARgAsAFwAbgAgACAAIAAgACgAUQAgACoAIABFAEMAIAAqACAARQBGACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAYwBvAG0AYgB1AHMAdABlAGQAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAAawBMAFwAbgBFAEMAIAA6ACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAOgAgAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBUAHIAYQBuAHMAdABxACwAIABFAEMAXwBUAHIAYQBuAHMAcQAsACAARQBGAF8AVAByAGEAbgBzADEAdABxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFQAcgBhAG4AcwB0AHEALAAgAEUAQwBfAFQAcgBhAG4AcwBxACwAIABFAEYAXwBUAHIAYQBuAHMAMQB0AHEAZwApAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsAVAByAGEAbgBzACwAdABxAH0AXABcAHQAaQBtAGUAcwAgAEUAQwBfAHsAVAByAGEAbgBzACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFQAcgBhAG4AcwAsADEALAB0AHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAFQAcgBhAG4AcwB0AHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIABjAG8AbQBiAHUAcwB0AGUAZAAgAGYAbwByACAAdAByAGEAbgBzAHAAbwByAHQAIABlAG4AZQByAGcAeQAgAHAAdQByAHAAbwBzAGUAcwBcACIALAAgAFwAIgBWAGEAcgBpAGUAcwAgAGIAYQBzAGUAZAAgAG8AbgAgAGYAdQBlAGwAIAB0AHkAcABlADoAIABrAEwALAAgAG0AMwAsACAARwBKAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAF8AVAByAGEAbgBzAHEAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AVAByAGEAbgBzADEAdABxAGcAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBcACIALAAgAFwAIgBGAHUAZQBsACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBcACIALAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwBcAG4AUQAgADoAIABBAG0AbwB1AG4AdAAgAG8AZgAgAGYAdQBlAGwAIAB0AHkAcABlACAAcQAgAHUAcwBlAGQAIABmAG8AcgAgAHMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBwAGUAcgBhAHQAaQBvAG4AcwAgADoAIABrAEwAXABuAEUAQwAgADoAIABFAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAEcASgAvAGsATABcAG4ARQBGACAAOgAgAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIAA6ACAAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AUwBDAHEALAAgAEUAQwBfAFMAQwBxACwAIABFAEYAXwBTAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFMAQwBxACwAIABFAEMAXwBTAEMAcQAsACAARQBGAF8AUwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAbwByACAAZQBhAGMAaAAgAEcASABHACAAZgByAG8AbQAgAHQAaABlACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdAAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AcQBcAFwAbABlAGYAdAAoAFEAXwB7AFMAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBDAF8AewBTAEMALABxAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUwBDACwAMQAsAHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AUwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAFMAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AUwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBDAFwAIgAsACAAXAAiAFMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADIAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBcAG4ARQBtAGkAcwBzAGkAbwBuAHMAIABmAG8AcgAgAGUAYQBjAGgAIABHAEgARwAgAGYAcgBvAG0AIABnAGUAbgBlAHIAaQBjACAAZgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIAB3AGgAZQByAGUAIAB0AGgAZQAgAHUAcwBhAGcAZQAgAGkAcwAgAG4AbwB0ACAAawBuAG8AdwBuAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAdQBzAGUAZAAgAGYAbwByACAAZwBlAG4AZQByAGkAYwAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAGsATABcAG4ARQBDACAAOgAgAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAGYAbwByACAAZQBhAGMAaAAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgADoAIABrAGcAIABDAE8AMgBlACAALwAgAEcASgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8ARwBDAHEALAAgAEUAQwBfAEcAQwBxACwAIABFAEYAXwBHAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAEcAQwBxACwAIABFAEMAXwBHAEMAcQAsACAARQBGAF8ARwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAG8AcgAgAGUAYQBjAGgAIABHAEgARwAgAGYAcgBvAG0AIAB0AGgAZQAgAGcAZQBuAGUAcgBpAGMAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVQBzAGUAcwAgAFYARQBFAFIARwAgADIAMAAyADYAOgAgADgALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApACwAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQAgAGEAbgBkACAAZQB2AGUAcgBhAGcAZQBzACAAdABoAGUAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGEAbgBkACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAZwBlAG4AZQByAGkAYwAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzACAAYQBuAGQAIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsARwBDACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEMAXwB7AEcAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBHAEMALAAxACwAcQBnAH0AXABcAHIAaQBnAGgAdAApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8ARwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAEcAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAGUAbgBlAHIAaQBjACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8ARwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwBlAG4AZQByAGkAYwAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBDAFwAIgAsACAAXAAiAEcAZQBuAGUAcgBpAGMAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAVABoAGkAcwAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAgAHUAcwBlAHMAIABhAHYAZQByAGEAZwBlAHMAIABvAGYAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGEAbgBkACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAdwBoAGUAcgBlACAAdABoAGUAIAB1AHMAYQBnAGUAIABpAHMAIABuAG8AdAAgAGsAbgBvAHcAbgAuAFwAIgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGEAdABhACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AE8AZgBmAFIAbwBhAGQAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEYAdQBlAGwAXwBHAGUAdABUAHIAYQBuAHMAcABvAHIAdABGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8ARwBlAHQAUwB0AGEAdABpAG8AbgBhAHIAeQBGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8AVABvAHQAYQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBVAG4AaQB0ACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVQBuAGkAdAAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -23012,24 +22789,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -23040,7 +22800,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23057,12 +22833,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>